<commit_message>
fix(excel): use English formula names and fix circular reference for openpyxl compatibility
</commit_message>
<xml_diff>
--- a/docs/examples/excel/cheatsheet_excel.xlsx
+++ b/docs/examples/excel/cheatsheet_excel.xlsx
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="K3" s="8">
-        <f>CONT.VALORES(A3:A54)</f>
+        <f>COUNTA(A3:A54)</f>
         <v/>
       </c>
     </row>
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="K4" s="8">
-        <f>CONT.SE(H3:H54,"Sim")</f>
+        <f>COUNTIF(H3:H54,"Sim")</f>
         <v/>
       </c>
     </row>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="K5" s="12">
-        <f>MEDIA(F3:F54)</f>
+        <f>AVERAGE(F3:F54)</f>
         <v/>
       </c>
     </row>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="K6" s="12">
-        <f>MAXIMO(F3:F54)</f>
+        <f>MAX(F3:F54)</f>
         <v/>
       </c>
     </row>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="K7" s="12">
-        <f>MINIMO(F3:F54)</f>
+        <f>MIN(F3:F54)</f>
         <v/>
       </c>
     </row>
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="K8" s="12">
-        <f>SOMA(F3:F54)</f>
+        <f>SUM(F3:F54)</f>
         <v/>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="K9" s="8">
-        <f>CONT.VALORES(F3:F54)-CONT.NUM(F3:F54)</f>
+        <f>COUNTA(F3:F54)-COUNT(F3:F54)</f>
         <v/>
       </c>
     </row>
@@ -2861,16 +2861,16 @@
         </is>
       </c>
       <c r="B3" s="16">
-        <f>CONT.SE(Dados!C3:C54,"TI")</f>
+        <f>COUNTIF(Dados!C3:C54,"TI")</f>
         <v/>
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>CONT.SES - TI E Ativo</t>
+          <t>COUNTIFS - TI E Ativo</t>
         </is>
       </c>
       <c r="F3" s="17">
-        <f>CONT.SES(Dados!C3:C54,"TI",Dados!H3:H54,"Sim")</f>
+        <f>COUNTIFS(Dados!C3:C54,"TI",Dados!H3:H54,"Sim")</f>
         <v/>
       </c>
     </row>
@@ -2881,16 +2881,16 @@
         </is>
       </c>
       <c r="B4" s="16">
-        <f>CONT.SE(Dados!H3:H54,"Sim")</f>
+        <f>COUNTIF(Dados!H3:H54,"Sim")</f>
         <v/>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>SOMASES - Vendas E Ativo</t>
+          <t>SUMIFS - Vendas E Ativo</t>
         </is>
       </c>
       <c r="F4" s="18">
-        <f>SOMASES(Dados!F3:F54,Dados!C3:C54,"Vendas",Dados!H3:H54,"Sim")</f>
+        <f>SUMIFS(Dados!F3:F54,Dados!C3:C54,"Vendas",Dados!H3:H54,"Sim")</f>
         <v/>
       </c>
     </row>
@@ -2901,16 +2901,16 @@
         </is>
       </c>
       <c r="B5" s="16">
-        <f>CONT.SE(Dados!F3:F54,"&gt;8000")</f>
+        <f>COUNTIF(Dados!F3:F54,"&gt;8000")</f>
         <v/>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>MEDIASES - TI E &gt; 5000</t>
+          <t>AVERAGEIFS - TI E &gt; 5000</t>
         </is>
       </c>
       <c r="F5" s="18">
-        <f>MEDIASES(Dados!F3:F54,Dados!C3:C54,"TI",Dados!F3:F54,"&gt;5000")</f>
+        <f>AVERAGEIFS(Dados!F3:F54,Dados!C3:C54,"TI",Dados!F3:F54,"&gt;5000")</f>
         <v/>
       </c>
     </row>
@@ -2921,7 +2921,7 @@
         </is>
       </c>
       <c r="B6" s="16">
-        <f>CONT.VALORES(Dados!F3:F54)-CONT.NUM(Dados!F3:F54)</f>
+        <f>COUNTA(Dados!F3:F54)-COUNT(Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -2930,7 +2930,7 @@
         </is>
       </c>
       <c r="F6" s="17">
-        <f>INDICE(Dados!B3:B54,CORRESP(MAXIMO(Dados!F3:F54),Dados!F3:F54,0))</f>
+        <f>INDEX(Dados!B3:B54,MATCH(MAX(Dados!F3:F54),Dados!F3:F54,0))</f>
         <v/>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
         </is>
       </c>
       <c r="B7" s="19">
-        <f>SOMASE(Dados!C3:C54,"TI",Dados!F3:F54)</f>
+        <f>SUMIF(Dados!C3:C54,"TI",Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -2950,7 +2950,7 @@
         </is>
       </c>
       <c r="F7" s="17">
-        <f>INDICE(Dados!B3:B54,CORRESP(MINIMO(Dados!F3:F54),Dados!F3:F54,0))</f>
+        <f>INDEX(Dados!B3:B54,MATCH(MIN(Dados!F3:F54),Dados!F3:F54,0))</f>
         <v/>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
         </is>
       </c>
       <c r="B8" s="19">
-        <f>SOMASE(Dados!F3:F54,"&gt;5000",Dados!F3:F54)</f>
+        <f>SUMIF(Dados!F3:F54,"&gt;5000",Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -2970,7 +2970,7 @@
         </is>
       </c>
       <c r="F8" s="18">
-        <f>GRANDE(Dados!F3:F54,3)</f>
+        <f>LARGE(Dados!F3:F54,3)</f>
         <v/>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="B9" s="19">
-        <f>MEDIASE(Dados!C3:C54,"TI",Dados!F3:F54)</f>
+        <f>AVERAGEIF(Dados!C3:C54,"TI",Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="E9" s="15" t="inlineStr">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="F9" s="18">
-        <f>PEQUENO(Dados!F3:F54,3)</f>
+        <f>SMALL(Dados!F3:F54,3)</f>
         <v/>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
         </is>
       </c>
       <c r="B10" s="19">
-        <f>MINIMO(Dados!F3:F54)</f>
+        <f>MIN(Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -3010,7 +3010,7 @@
         </is>
       </c>
       <c r="F10" s="18">
-        <f>SOMARPRODUTO(1/CONT.SE(Dados!C3:C53,Dados!C3:C53))</f>
+        <f>SUMRPRODUTO(1/COUNTIF(Dados!C3:C53,Dados!C3:C53))</f>
         <v/>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
         </is>
       </c>
       <c r="B11" s="19">
-        <f>MAXIMO(Dados!F3:F54)</f>
+        <f>MAX(Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -3030,7 +3030,7 @@
         </is>
       </c>
       <c r="F11" s="20">
-        <f>CONT.SE(Dados!F3:F54,"&gt;8000")/CONT.VALORES(Dados!F3:F54)</f>
+        <f>COUNTIF(Dados!F3:F54,"&gt;8000")/COUNTA(Dados!F3:F54)</f>
         <v/>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
         </is>
       </c>
       <c r="B12" s="19">
-        <f>SOMA(Dados!F3:F54)</f>
+        <f>SUM(Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -3050,7 +3050,7 @@
         </is>
       </c>
       <c r="F12" s="18">
-        <f>SOMASE(Dados!H3:H54,"Sim",Dados!F3:F54)</f>
+        <f>SUMIF(Dados!H3:H54,"Sim",Dados!F3:F54)</f>
         <v/>
       </c>
     </row>
@@ -3138,23 +3138,23 @@
         </is>
       </c>
       <c r="B3" s="24">
-        <f>CONT.SE(Dados!C$3:C$54,A3)</f>
+        <f>COUNTIF(Dados!C$3:C$54,A3)</f>
         <v/>
       </c>
       <c r="C3" s="25">
-        <f>SOMASE(Dados!C$3:C$54,A3,Dados!F$3:F$54)</f>
+        <f>SUMIF(Dados!C$3:C$54,A3,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="D3" s="25">
-        <f>MEDIASE(Dados!C$3:C$54,A3,Dados!F$3:F$54)</f>
+        <f>AVERAGEIF(Dados!C$3:C$54,A3,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="E3" s="25">
-        <f>MAXSES(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
+        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
         <v/>
       </c>
       <c r="F3" s="25">
-        <f>MINSES(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
+        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
         <v/>
       </c>
       <c r="G3" s="26">
@@ -3169,23 +3169,23 @@
         </is>
       </c>
       <c r="B4" s="24">
-        <f>CONT.SE(Dados!C$3:C$54,A4)</f>
+        <f>COUNTIF(Dados!C$3:C$54,A4)</f>
         <v/>
       </c>
       <c r="C4" s="25">
-        <f>SOMASE(Dados!C$3:C$54,A4,Dados!F$3:F$54)</f>
+        <f>SUMIF(Dados!C$3:C$54,A4,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="D4" s="25">
-        <f>MEDIASE(Dados!C$3:C$54,A4,Dados!F$3:F$54)</f>
+        <f>AVERAGEIF(Dados!C$3:C$54,A4,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="E4" s="25">
-        <f>MAXSES(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
+        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
         <v/>
       </c>
       <c r="F4" s="25">
-        <f>MINSES(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
+        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
         <v/>
       </c>
       <c r="G4" s="26">
@@ -3200,23 +3200,23 @@
         </is>
       </c>
       <c r="B5" s="24">
-        <f>CONT.SE(Dados!C$3:C$54,A5)</f>
+        <f>COUNTIF(Dados!C$3:C$54,A5)</f>
         <v/>
       </c>
       <c r="C5" s="25">
-        <f>SOMASE(Dados!C$3:C$54,A5,Dados!F$3:F$54)</f>
+        <f>SUMIF(Dados!C$3:C$54,A5,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="D5" s="25">
-        <f>MEDIASE(Dados!C$3:C$54,A5,Dados!F$3:F$54)</f>
+        <f>AVERAGEIF(Dados!C$3:C$54,A5,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="E5" s="25">
-        <f>MAXSES(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
+        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
         <v/>
       </c>
       <c r="F5" s="25">
-        <f>MINSES(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
+        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
         <v/>
       </c>
       <c r="G5" s="26">
@@ -3231,23 +3231,23 @@
         </is>
       </c>
       <c r="B6" s="24">
-        <f>CONT.SE(Dados!C$3:C$54,A6)</f>
+        <f>COUNTIF(Dados!C$3:C$54,A6)</f>
         <v/>
       </c>
       <c r="C6" s="25">
-        <f>SOMASE(Dados!C$3:C$54,A6,Dados!F$3:F$54)</f>
+        <f>SUMIF(Dados!C$3:C$54,A6,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="D6" s="25">
-        <f>MEDIASE(Dados!C$3:C$54,A6,Dados!F$3:F$54)</f>
+        <f>AVERAGEIF(Dados!C$3:C$54,A6,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="E6" s="25">
-        <f>MAXSES(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
+        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
         <v/>
       </c>
       <c r="F6" s="25">
-        <f>MINSES(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
+        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
         <v/>
       </c>
       <c r="G6" s="26">
@@ -3262,23 +3262,23 @@
         </is>
       </c>
       <c r="B7" s="24">
-        <f>CONT.SE(Dados!C$3:C$54,A7)</f>
+        <f>COUNTIF(Dados!C$3:C$54,A7)</f>
         <v/>
       </c>
       <c r="C7" s="25">
-        <f>SOMASE(Dados!C$3:C$54,A7,Dados!F$3:F$54)</f>
+        <f>SUMIF(Dados!C$3:C$54,A7,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="D7" s="25">
-        <f>MEDIASE(Dados!C$3:C$54,A7,Dados!F$3:F$54)</f>
+        <f>AVERAGEIF(Dados!C$3:C$54,A7,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="E7" s="25">
-        <f>MAXSES(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
+        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
         <v/>
       </c>
       <c r="F7" s="25">
-        <f>MINSES(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
+        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
         <v/>
       </c>
       <c r="G7" s="26">
@@ -3293,23 +3293,23 @@
         </is>
       </c>
       <c r="B8" s="24">
-        <f>CONT.SE(Dados!C$3:C$54,A8)</f>
+        <f>COUNTIF(Dados!C$3:C$54,A8)</f>
         <v/>
       </c>
       <c r="C8" s="25">
-        <f>SOMASE(Dados!C$3:C$54,A8,Dados!F$3:F$54)</f>
+        <f>SUMIF(Dados!C$3:C$54,A8,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="D8" s="25">
-        <f>MEDIASE(Dados!C$3:C$54,A8,Dados!F$3:F$54)</f>
+        <f>AVERAGEIF(Dados!C$3:C$54,A8,Dados!F$3:F$54)</f>
         <v/>
       </c>
       <c r="E8" s="25">
-        <f>MAXSES(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
+        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
         <v/>
       </c>
       <c r="F8" s="25">
-        <f>MINSES(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
+        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
         <v/>
       </c>
       <c r="G8" s="26">
@@ -3324,34 +3324,34 @@
         </is>
       </c>
       <c r="B9" s="29">
-        <f>SOMA(B3:B8)</f>
+        <f>SUM(B3:B8)</f>
         <v/>
       </c>
       <c r="C9" s="30">
-        <f>SOMA(C3:C8)</f>
+        <f>SUM(C3:C8)</f>
         <v/>
       </c>
       <c r="D9" s="30">
-        <f>MEDIA(Dados!F3:F54)</f>
+        <f>AVERAGE(Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="E9" s="30">
-        <f>MAXIMO(Dados!F3:F54)</f>
+        <f>MAX(Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="F9" s="30">
-        <f>MINIMO(Dados!F3:F54)</f>
+        <f>MIN(Dados!F3:F54)</f>
         <v/>
       </c>
       <c r="G9" s="31">
-        <f>SOMA(G3:G8)</f>
+        <f>SUM(G3:G8)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>Nota: MAXSES e MINSES requerem Excel 2019 ou 365. Em versoes mais antigas, use MAXIMO com SEERRO(INDICE...)</t>
+          <t>Nota: MAXIFS e MINIFS requerem Excel 2019 ou 365. Em versoes mais antigas, use MAX com IFERROR(INDEX...)</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="B3" s="16">
-        <f>ANO(Dados!G3)</f>
+        <f>YEAR(Dados!G3)</f>
         <v/>
       </c>
       <c r="E3" s="15" t="inlineStr">
@@ -3426,7 +3426,7 @@
         </is>
       </c>
       <c r="F3" s="17">
-        <f>HOJE()-Dados!G3</f>
+        <f>TODAY()-Dados!G3</f>
         <v/>
       </c>
     </row>
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="B4" s="16">
-        <f>MES(Dados!G3)</f>
+        <f>MONTH(Dados!G3)</f>
         <v/>
       </c>
       <c r="E4" s="15" t="inlineStr">
@@ -3446,7 +3446,7 @@
         </is>
       </c>
       <c r="F4" s="32">
-        <f>FRAÇÃO.ANO(Dados!G3,HOJE())</f>
+        <f>FRAÇÃO.YEAR(Dados!G3,TODAY())</f>
         <v/>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="B5" s="16">
-        <f>DIA(Dados!G3)</f>
+        <f>DAY(Dados!G3)</f>
         <v/>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -3466,7 +3466,7 @@
         </is>
       </c>
       <c r="F5" s="17">
-        <f>DATAM(Dados!G3,0)</f>
+        <f>EDATE(Dados!G3,0)</f>
         <v/>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
         </is>
       </c>
       <c r="B6" s="16">
-        <f>TEXTO(Dados!G3,"MMMM")</f>
+        <f>TEXT(Dados!G3,"MMMM")</f>
         <v/>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>TEXTO(Dados!G3,"DDDD")</f>
+        <f>TEXT(Dados!G3,"DDDD")</f>
         <v/>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -3506,7 +3506,7 @@
         </is>
       </c>
       <c r="F7" s="17">
-        <f>DATA(ANO(Dados!G3),MES(Dados!G3),1)</f>
+        <f>DATE(YEAR(Dados!G3),MONTH(Dados!G3),1)</f>
         <v/>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
         </is>
       </c>
       <c r="B8" s="16">
-        <f>DIA.DA.SEMANA(Dados!G3,2)</f>
+        <f>WEEKDAY(Dados!G3,2)</f>
         <v/>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -3526,7 +3526,7 @@
         </is>
       </c>
       <c r="F8" s="17">
-        <f>FIMMÊS(Dados!G3,0)</f>
+        <f>EOMONTH(Dados!G3,0)</f>
         <v/>
       </c>
     </row>
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="B9" s="16">
-        <f>INT((MES(Dados!G3)-1)/3)+1</f>
+        <f>INT((MONTH(Dados!G3)-1)/3)+1</f>
         <v/>
       </c>
       <c r="E9" s="15" t="inlineStr">
@@ -3546,7 +3546,7 @@
         </is>
       </c>
       <c r="F9" s="33">
-        <f>DIAS(HOJE(),Dados!G3)</f>
+        <f>DAYS(TODAY(),Dados!G3)</f>
         <v/>
       </c>
     </row>
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="B10" s="16">
-        <f>NUM.SEMANA(Dados!G3,2)</f>
+        <f>WEEKNUM(Dados!G3,2)</f>
         <v/>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -3566,7 +3566,7 @@
         </is>
       </c>
       <c r="F10" s="33">
-        <f>DIATRABALHO(Dados!G3,30)</f>
+        <f>WORKDAY(Dados!G3,30)</f>
         <v/>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="B11" s="34">
-        <f>HOJE()</f>
+        <f>TODAY()</f>
         <v/>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -3586,7 +3586,7 @@
         </is>
       </c>
       <c r="F11" s="17">
-        <f>CONT.SE(Dados!G3:G54,"&gt;=01/01/2023")-CONT.SE(Dados!G3:G54,"&gt;=01/01/2024")</f>
+        <f>COUNTIF(Dados!G3:G54,"&gt;=01/01/2023")-COUNTIF(Dados!G3:G54,"&gt;=01/01/2024")</f>
         <v/>
       </c>
     </row>
@@ -3597,7 +3597,7 @@
         </is>
       </c>
       <c r="B12" s="35">
-        <f>AGORA()</f>
+        <f>NOW()</f>
         <v/>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -3606,7 +3606,7 @@
         </is>
       </c>
       <c r="F12" s="33">
-        <f>MAXIMO(Dados!G3:G54)</f>
+        <f>MAX(Dados!G3:G54)</f>
         <v/>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>Coluna Condicional — SE, IFS, SEERRO, SWITCH</t>
+          <t>Coluna Condicional — SE, IFS, IFERROR, SWITCH</t>
         </is>
       </c>
     </row>
@@ -3695,19 +3695,19 @@
         <v>2955.07</v>
       </c>
       <c r="D3" s="39">
-        <f>SE(C3&gt;12000,"Especialista",SE(C3&gt;8000,"Senior",SE(C3&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C3&gt;12000,"Especialista",IF(C3&gt;8000,"Senior",IF(C3&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E3" s="39">
-        <f>IFS(C3&gt;12000,"Especialista",C3&gt;8000,"Senior",C3&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C3&gt;12000,"Especialista",C3&gt;8000,"Senior",C3&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F3" s="40">
-        <f>SE(C3&gt;10000,"Alto",SE(C3&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C3&gt;10000,"Alto",IF(C3&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G3" s="40">
-        <f>SE(G3="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H3="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3722,19 +3722,19 @@
         <v>4842.67</v>
       </c>
       <c r="D4" s="39">
-        <f>SE(C4&gt;12000,"Especialista",SE(C4&gt;8000,"Senior",SE(C4&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C4&gt;12000,"Especialista",IF(C4&gt;8000,"Senior",IF(C4&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E4" s="39">
-        <f>IFS(C4&gt;12000,"Especialista",C4&gt;8000,"Senior",C4&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C4&gt;12000,"Especialista",C4&gt;8000,"Senior",C4&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F4" s="40">
-        <f>SE(C4&gt;10000,"Alto",SE(C4&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C4&gt;10000,"Alto",IF(C4&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G4" s="40">
-        <f>SE(G4="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H4="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3753,19 +3753,19 @@
         <v>8303.389999999999</v>
       </c>
       <c r="D5" s="39">
-        <f>SE(C5&gt;12000,"Especialista",SE(C5&gt;8000,"Senior",SE(C5&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C5&gt;12000,"Especialista",IF(C5&gt;8000,"Senior",IF(C5&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E5" s="39">
-        <f>IFS(C5&gt;12000,"Especialista",C5&gt;8000,"Senior",C5&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C5&gt;12000,"Especialista",C5&gt;8000,"Senior",C5&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F5" s="40">
-        <f>SE(C5&gt;10000,"Alto",SE(C5&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C5&gt;10000,"Alto",IF(C5&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G5" s="40">
-        <f>SE(G5="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H5="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3784,19 +3784,19 @@
         <v>4102.85</v>
       </c>
       <c r="D6" s="39">
-        <f>SE(C6&gt;12000,"Especialista",SE(C6&gt;8000,"Senior",SE(C6&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C6&gt;12000,"Especialista",IF(C6&gt;8000,"Senior",IF(C6&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E6" s="39">
-        <f>IFS(C6&gt;12000,"Especialista",C6&gt;8000,"Senior",C6&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C6&gt;12000,"Especialista",C6&gt;8000,"Senior",C6&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F6" s="40">
-        <f>SE(C6&gt;10000,"Alto",SE(C6&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C6&gt;10000,"Alto",IF(C6&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G6" s="40">
-        <f>SE(G6="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H6="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3813,19 +3813,19 @@
       </c>
       <c r="C7" s="38" t="n"/>
       <c r="D7" s="39">
-        <f>SE(C7&gt;12000,"Especialista",SE(C7&gt;8000,"Senior",SE(C7&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C7&gt;12000,"Especialista",IF(C7&gt;8000,"Senior",IF(C7&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E7" s="39">
-        <f>IFS(C7&gt;12000,"Especialista",C7&gt;8000,"Senior",C7&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C7&gt;12000,"Especialista",C7&gt;8000,"Senior",C7&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F7" s="40">
-        <f>SE(C7&gt;10000,"Alto",SE(C7&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C7&gt;10000,"Alto",IF(C7&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G7" s="40">
-        <f>SE(G7="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H7="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3844,19 +3844,19 @@
         <v>9059.57</v>
       </c>
       <c r="D8" s="39">
-        <f>SE(C8&gt;12000,"Especialista",SE(C8&gt;8000,"Senior",SE(C8&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C8&gt;12000,"Especialista",IF(C8&gt;8000,"Senior",IF(C8&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E8" s="39">
-        <f>IFS(C8&gt;12000,"Especialista",C8&gt;8000,"Senior",C8&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C8&gt;12000,"Especialista",C8&gt;8000,"Senior",C8&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F8" s="40">
-        <f>SE(C8&gt;10000,"Alto",SE(C8&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C8&gt;10000,"Alto",IF(C8&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G8" s="40">
-        <f>SE(G8="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H8="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3875,19 +3875,19 @@
         <v>7459.35</v>
       </c>
       <c r="D9" s="39">
-        <f>SE(C9&gt;12000,"Especialista",SE(C9&gt;8000,"Senior",SE(C9&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C9&gt;12000,"Especialista",IF(C9&gt;8000,"Senior",IF(C9&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E9" s="39">
-        <f>IFS(C9&gt;12000,"Especialista",C9&gt;8000,"Senior",C9&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C9&gt;12000,"Especialista",C9&gt;8000,"Senior",C9&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F9" s="40">
-        <f>SE(C9&gt;10000,"Alto",SE(C9&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C9&gt;10000,"Alto",IF(C9&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G9" s="40">
-        <f>SE(G9="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H9="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3904,19 +3904,19 @@
       </c>
       <c r="C10" s="42" t="n"/>
       <c r="D10" s="39">
-        <f>SE(C10&gt;12000,"Especialista",SE(C10&gt;8000,"Senior",SE(C10&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C10&gt;12000,"Especialista",IF(C10&gt;8000,"Senior",IF(C10&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E10" s="39">
-        <f>IFS(C10&gt;12000,"Especialista",C10&gt;8000,"Senior",C10&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C10&gt;12000,"Especialista",C10&gt;8000,"Senior",C10&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F10" s="40">
-        <f>SE(C10&gt;10000,"Alto",SE(C10&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C10&gt;10000,"Alto",IF(C10&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G10" s="40">
-        <f>SE(G10="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H10="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3935,19 +3935,19 @@
         <v>4701.01</v>
       </c>
       <c r="D11" s="39">
-        <f>SE(C11&gt;12000,"Especialista",SE(C11&gt;8000,"Senior",SE(C11&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C11&gt;12000,"Especialista",IF(C11&gt;8000,"Senior",IF(C11&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E11" s="39">
-        <f>IFS(C11&gt;12000,"Especialista",C11&gt;8000,"Senior",C11&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C11&gt;12000,"Especialista",C11&gt;8000,"Senior",C11&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F11" s="40">
-        <f>SE(C11&gt;10000,"Alto",SE(C11&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C11&gt;10000,"Alto",IF(C11&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G11" s="40">
-        <f>SE(G11="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H11="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3964,19 +3964,19 @@
       </c>
       <c r="C12" s="42" t="n"/>
       <c r="D12" s="39">
-        <f>SE(C12&gt;12000,"Especialista",SE(C12&gt;8000,"Senior",SE(C12&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C12&gt;12000,"Especialista",IF(C12&gt;8000,"Senior",IF(C12&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E12" s="39">
-        <f>IFS(C12&gt;12000,"Especialista",C12&gt;8000,"Senior",C12&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C12&gt;12000,"Especialista",C12&gt;8000,"Senior",C12&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F12" s="40">
-        <f>SE(C12&gt;10000,"Alto",SE(C12&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C12&gt;10000,"Alto",IF(C12&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G12" s="40">
-        <f>SE(G12="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H12="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -3995,19 +3995,19 @@
         <v>7710.89</v>
       </c>
       <c r="D13" s="39">
-        <f>SE(C13&gt;12000,"Especialista",SE(C13&gt;8000,"Senior",SE(C13&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C13&gt;12000,"Especialista",IF(C13&gt;8000,"Senior",IF(C13&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E13" s="39">
-        <f>IFS(C13&gt;12000,"Especialista",C13&gt;8000,"Senior",C13&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C13&gt;12000,"Especialista",C13&gt;8000,"Senior",C13&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F13" s="40">
-        <f>SE(C13&gt;10000,"Alto",SE(C13&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C13&gt;10000,"Alto",IF(C13&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G13" s="40">
-        <f>SE(G13="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H13="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4026,19 +4026,19 @@
         <v>13862.23</v>
       </c>
       <c r="D14" s="39">
-        <f>SE(C14&gt;12000,"Especialista",SE(C14&gt;8000,"Senior",SE(C14&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C14&gt;12000,"Especialista",IF(C14&gt;8000,"Senior",IF(C14&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E14" s="39">
-        <f>IFS(C14&gt;12000,"Especialista",C14&gt;8000,"Senior",C14&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C14&gt;12000,"Especialista",C14&gt;8000,"Senior",C14&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F14" s="40">
-        <f>SE(C14&gt;10000,"Alto",SE(C14&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C14&gt;10000,"Alto",IF(C14&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G14" s="40">
-        <f>SE(G14="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H14="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4057,19 +4057,19 @@
         <v>8825.709999999999</v>
       </c>
       <c r="D15" s="39">
-        <f>SE(C15&gt;12000,"Especialista",SE(C15&gt;8000,"Senior",SE(C15&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C15&gt;12000,"Especialista",IF(C15&gt;8000,"Senior",IF(C15&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E15" s="39">
-        <f>IFS(C15&gt;12000,"Especialista",C15&gt;8000,"Senior",C15&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C15&gt;12000,"Especialista",C15&gt;8000,"Senior",C15&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F15" s="40">
-        <f>SE(C15&gt;10000,"Alto",SE(C15&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C15&gt;10000,"Alto",IF(C15&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G15" s="40">
-        <f>SE(G15="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H15="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4088,19 +4088,19 @@
         <v>9862.6</v>
       </c>
       <c r="D16" s="39">
-        <f>SE(C16&gt;12000,"Especialista",SE(C16&gt;8000,"Senior",SE(C16&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C16&gt;12000,"Especialista",IF(C16&gt;8000,"Senior",IF(C16&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E16" s="39">
-        <f>IFS(C16&gt;12000,"Especialista",C16&gt;8000,"Senior",C16&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C16&gt;12000,"Especialista",C16&gt;8000,"Senior",C16&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F16" s="40">
-        <f>SE(C16&gt;10000,"Alto",SE(C16&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C16&gt;10000,"Alto",IF(C16&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G16" s="40">
-        <f>SE(G16="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H16="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4117,19 +4117,19 @@
       </c>
       <c r="C17" s="38" t="n"/>
       <c r="D17" s="39">
-        <f>SE(C17&gt;12000,"Especialista",SE(C17&gt;8000,"Senior",SE(C17&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C17&gt;12000,"Especialista",IF(C17&gt;8000,"Senior",IF(C17&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E17" s="39">
-        <f>IFS(C17&gt;12000,"Especialista",C17&gt;8000,"Senior",C17&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C17&gt;12000,"Especialista",C17&gt;8000,"Senior",C17&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F17" s="40">
-        <f>SE(C17&gt;10000,"Alto",SE(C17&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C17&gt;10000,"Alto",IF(C17&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G17" s="40">
-        <f>SE(G17="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H17="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4148,19 +4148,19 @@
         <v>8937.76</v>
       </c>
       <c r="D18" s="39">
-        <f>SE(C18&gt;12000,"Especialista",SE(C18&gt;8000,"Senior",SE(C18&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C18&gt;12000,"Especialista",IF(C18&gt;8000,"Senior",IF(C18&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E18" s="39">
-        <f>IFS(C18&gt;12000,"Especialista",C18&gt;8000,"Senior",C18&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C18&gt;12000,"Especialista",C18&gt;8000,"Senior",C18&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F18" s="40">
-        <f>SE(C18&gt;10000,"Alto",SE(C18&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C18&gt;10000,"Alto",IF(C18&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G18" s="40">
-        <f>SE(G18="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H18="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4179,19 +4179,19 @@
         <v>7220.28</v>
       </c>
       <c r="D19" s="39">
-        <f>SE(C19&gt;12000,"Especialista",SE(C19&gt;8000,"Senior",SE(C19&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C19&gt;12000,"Especialista",IF(C19&gt;8000,"Senior",IF(C19&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E19" s="39">
-        <f>IFS(C19&gt;12000,"Especialista",C19&gt;8000,"Senior",C19&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C19&gt;12000,"Especialista",C19&gt;8000,"Senior",C19&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F19" s="40">
-        <f>SE(C19&gt;10000,"Alto",SE(C19&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C19&gt;10000,"Alto",IF(C19&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G19" s="40">
-        <f>SE(G19="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H19="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4206,19 +4206,19 @@
         <v>7324.01</v>
       </c>
       <c r="D20" s="39">
-        <f>SE(C20&gt;12000,"Especialista",SE(C20&gt;8000,"Senior",SE(C20&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C20&gt;12000,"Especialista",IF(C20&gt;8000,"Senior",IF(C20&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E20" s="39">
-        <f>IFS(C20&gt;12000,"Especialista",C20&gt;8000,"Senior",C20&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C20&gt;12000,"Especialista",C20&gt;8000,"Senior",C20&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F20" s="40">
-        <f>SE(C20&gt;10000,"Alto",SE(C20&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C20&gt;10000,"Alto",IF(C20&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G20" s="40">
-        <f>SE(G20="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H20="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4237,19 +4237,19 @@
         <v>6842.01</v>
       </c>
       <c r="D21" s="39">
-        <f>SE(C21&gt;12000,"Especialista",SE(C21&gt;8000,"Senior",SE(C21&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C21&gt;12000,"Especialista",IF(C21&gt;8000,"Senior",IF(C21&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E21" s="39">
-        <f>IFS(C21&gt;12000,"Especialista",C21&gt;8000,"Senior",C21&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C21&gt;12000,"Especialista",C21&gt;8000,"Senior",C21&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F21" s="40">
-        <f>SE(C21&gt;10000,"Alto",SE(C21&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C21&gt;10000,"Alto",IF(C21&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G21" s="40">
-        <f>SE(G21="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H21="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4268,19 +4268,19 @@
         <v>10267.47</v>
       </c>
       <c r="D22" s="39">
-        <f>SE(C22&gt;12000,"Especialista",SE(C22&gt;8000,"Senior",SE(C22&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C22&gt;12000,"Especialista",IF(C22&gt;8000,"Senior",IF(C22&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E22" s="39">
-        <f>IFS(C22&gt;12000,"Especialista",C22&gt;8000,"Senior",C22&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C22&gt;12000,"Especialista",C22&gt;8000,"Senior",C22&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F22" s="40">
-        <f>SE(C22&gt;10000,"Alto",SE(C22&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C22&gt;10000,"Alto",IF(C22&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G22" s="40">
-        <f>SE(G22="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H22="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4299,19 +4299,19 @@
         <v>3175.8</v>
       </c>
       <c r="D23" s="39">
-        <f>SE(C23&gt;12000,"Especialista",SE(C23&gt;8000,"Senior",SE(C23&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C23&gt;12000,"Especialista",IF(C23&gt;8000,"Senior",IF(C23&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E23" s="39">
-        <f>IFS(C23&gt;12000,"Especialista",C23&gt;8000,"Senior",C23&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C23&gt;12000,"Especialista",C23&gt;8000,"Senior",C23&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F23" s="40">
-        <f>SE(C23&gt;10000,"Alto",SE(C23&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C23&gt;10000,"Alto",IF(C23&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G23" s="40">
-        <f>SE(G23="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H23="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4330,19 +4330,19 @@
         <v>5123.74</v>
       </c>
       <c r="D24" s="39">
-        <f>SE(C24&gt;12000,"Especialista",SE(C24&gt;8000,"Senior",SE(C24&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C24&gt;12000,"Especialista",IF(C24&gt;8000,"Senior",IF(C24&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E24" s="39">
-        <f>IFS(C24&gt;12000,"Especialista",C24&gt;8000,"Senior",C24&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C24&gt;12000,"Especialista",C24&gt;8000,"Senior",C24&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F24" s="40">
-        <f>SE(C24&gt;10000,"Alto",SE(C24&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C24&gt;10000,"Alto",IF(C24&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G24" s="40">
-        <f>SE(G24="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H24="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4359,19 +4359,19 @@
       </c>
       <c r="C25" s="38" t="n"/>
       <c r="D25" s="39">
-        <f>SE(C25&gt;12000,"Especialista",SE(C25&gt;8000,"Senior",SE(C25&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C25&gt;12000,"Especialista",IF(C25&gt;8000,"Senior",IF(C25&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E25" s="39">
-        <f>IFS(C25&gt;12000,"Especialista",C25&gt;8000,"Senior",C25&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C25&gt;12000,"Especialista",C25&gt;8000,"Senior",C25&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F25" s="40">
-        <f>SE(C25&gt;10000,"Alto",SE(C25&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C25&gt;10000,"Alto",IF(C25&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G25" s="40">
-        <f>SE(G25="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H25="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4390,19 +4390,19 @@
         <v>9364.59</v>
       </c>
       <c r="D26" s="39">
-        <f>SE(C26&gt;12000,"Especialista",SE(C26&gt;8000,"Senior",SE(C26&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C26&gt;12000,"Especialista",IF(C26&gt;8000,"Senior",IF(C26&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E26" s="39">
-        <f>IFS(C26&gt;12000,"Especialista",C26&gt;8000,"Senior",C26&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C26&gt;12000,"Especialista",C26&gt;8000,"Senior",C26&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F26" s="40">
-        <f>SE(C26&gt;10000,"Alto",SE(C26&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C26&gt;10000,"Alto",IF(C26&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G26" s="40">
-        <f>SE(G26="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H26="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4421,19 +4421,19 @@
         <v>8983.799999999999</v>
       </c>
       <c r="D27" s="39">
-        <f>SE(C27&gt;12000,"Especialista",SE(C27&gt;8000,"Senior",SE(C27&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C27&gt;12000,"Especialista",IF(C27&gt;8000,"Senior",IF(C27&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E27" s="39">
-        <f>IFS(C27&gt;12000,"Especialista",C27&gt;8000,"Senior",C27&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C27&gt;12000,"Especialista",C27&gt;8000,"Senior",C27&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F27" s="40">
-        <f>SE(C27&gt;10000,"Alto",SE(C27&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C27&gt;10000,"Alto",IF(C27&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G27" s="40">
-        <f>SE(G27="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H27="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4452,19 +4452,19 @@
         <v>5890.78</v>
       </c>
       <c r="D28" s="39">
-        <f>SE(C28&gt;12000,"Especialista",SE(C28&gt;8000,"Senior",SE(C28&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C28&gt;12000,"Especialista",IF(C28&gt;8000,"Senior",IF(C28&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E28" s="39">
-        <f>IFS(C28&gt;12000,"Especialista",C28&gt;8000,"Senior",C28&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C28&gt;12000,"Especialista",C28&gt;8000,"Senior",C28&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F28" s="40">
-        <f>SE(C28&gt;10000,"Alto",SE(C28&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C28&gt;10000,"Alto",IF(C28&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G28" s="40">
-        <f>SE(G28="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H28="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4483,19 +4483,19 @@
         <v>10449.92</v>
       </c>
       <c r="D29" s="39">
-        <f>SE(C29&gt;12000,"Especialista",SE(C29&gt;8000,"Senior",SE(C29&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C29&gt;12000,"Especialista",IF(C29&gt;8000,"Senior",IF(C29&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E29" s="39">
-        <f>IFS(C29&gt;12000,"Especialista",C29&gt;8000,"Senior",C29&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C29&gt;12000,"Especialista",C29&gt;8000,"Senior",C29&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F29" s="40">
-        <f>SE(C29&gt;10000,"Alto",SE(C29&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C29&gt;10000,"Alto",IF(C29&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G29" s="40">
-        <f>SE(G29="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H29="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4510,19 +4510,19 @@
         <v>12224.44</v>
       </c>
       <c r="D30" s="39">
-        <f>SE(C30&gt;12000,"Especialista",SE(C30&gt;8000,"Senior",SE(C30&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C30&gt;12000,"Especialista",IF(C30&gt;8000,"Senior",IF(C30&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E30" s="39">
-        <f>IFS(C30&gt;12000,"Especialista",C30&gt;8000,"Senior",C30&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C30&gt;12000,"Especialista",C30&gt;8000,"Senior",C30&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F30" s="40">
-        <f>SE(C30&gt;10000,"Alto",SE(C30&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C30&gt;10000,"Alto",IF(C30&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G30" s="40">
-        <f>SE(G30="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H30="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4541,19 +4541,19 @@
         <v>7047.08</v>
       </c>
       <c r="D31" s="39">
-        <f>SE(C31&gt;12000,"Especialista",SE(C31&gt;8000,"Senior",SE(C31&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C31&gt;12000,"Especialista",IF(C31&gt;8000,"Senior",IF(C31&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E31" s="39">
-        <f>IFS(C31&gt;12000,"Especialista",C31&gt;8000,"Senior",C31&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C31&gt;12000,"Especialista",C31&gt;8000,"Senior",C31&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F31" s="40">
-        <f>SE(C31&gt;10000,"Alto",SE(C31&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C31&gt;10000,"Alto",IF(C31&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G31" s="40">
-        <f>SE(G31="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H31="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4572,19 +4572,19 @@
         <v>6592.4</v>
       </c>
       <c r="D32" s="39">
-        <f>SE(C32&gt;12000,"Especialista",SE(C32&gt;8000,"Senior",SE(C32&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C32&gt;12000,"Especialista",IF(C32&gt;8000,"Senior",IF(C32&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E32" s="39">
-        <f>IFS(C32&gt;12000,"Especialista",C32&gt;8000,"Senior",C32&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C32&gt;12000,"Especialista",C32&gt;8000,"Senior",C32&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F32" s="40">
-        <f>SE(C32&gt;10000,"Alto",SE(C32&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C32&gt;10000,"Alto",IF(C32&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G32" s="40">
-        <f>SE(G32="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H32="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4603,19 +4603,19 @@
         <v>14651.42</v>
       </c>
       <c r="D33" s="39">
-        <f>SE(C33&gt;12000,"Especialista",SE(C33&gt;8000,"Senior",SE(C33&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C33&gt;12000,"Especialista",IF(C33&gt;8000,"Senior",IF(C33&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E33" s="39">
-        <f>IFS(C33&gt;12000,"Especialista",C33&gt;8000,"Senior",C33&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C33&gt;12000,"Especialista",C33&gt;8000,"Senior",C33&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F33" s="40">
-        <f>SE(C33&gt;10000,"Alto",SE(C33&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C33&gt;10000,"Alto",IF(C33&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G33" s="40">
-        <f>SE(G33="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H33="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4634,19 +4634,19 @@
         <v>5008.97</v>
       </c>
       <c r="D34" s="39">
-        <f>SE(C34&gt;12000,"Especialista",SE(C34&gt;8000,"Senior",SE(C34&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C34&gt;12000,"Especialista",IF(C34&gt;8000,"Senior",IF(C34&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E34" s="39">
-        <f>IFS(C34&gt;12000,"Especialista",C34&gt;8000,"Senior",C34&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C34&gt;12000,"Especialista",C34&gt;8000,"Senior",C34&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F34" s="40">
-        <f>SE(C34&gt;10000,"Alto",SE(C34&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C34&gt;10000,"Alto",IF(C34&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G34" s="40">
-        <f>SE(G34="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H34="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4661,19 +4661,19 @@
         <v>8318</v>
       </c>
       <c r="D35" s="39">
-        <f>SE(C35&gt;12000,"Especialista",SE(C35&gt;8000,"Senior",SE(C35&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C35&gt;12000,"Especialista",IF(C35&gt;8000,"Senior",IF(C35&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E35" s="39">
-        <f>IFS(C35&gt;12000,"Especialista",C35&gt;8000,"Senior",C35&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C35&gt;12000,"Especialista",C35&gt;8000,"Senior",C35&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F35" s="40">
-        <f>SE(C35&gt;10000,"Alto",SE(C35&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C35&gt;10000,"Alto",IF(C35&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G35" s="40">
-        <f>SE(G35="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H35="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4692,19 +4692,19 @@
         <v>9676.76</v>
       </c>
       <c r="D36" s="39">
-        <f>SE(C36&gt;12000,"Especialista",SE(C36&gt;8000,"Senior",SE(C36&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C36&gt;12000,"Especialista",IF(C36&gt;8000,"Senior",IF(C36&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E36" s="39">
-        <f>IFS(C36&gt;12000,"Especialista",C36&gt;8000,"Senior",C36&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C36&gt;12000,"Especialista",C36&gt;8000,"Senior",C36&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F36" s="40">
-        <f>SE(C36&gt;10000,"Alto",SE(C36&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C36&gt;10000,"Alto",IF(C36&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G36" s="40">
-        <f>SE(G36="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H36="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4723,19 +4723,19 @@
         <v>7730.99</v>
       </c>
       <c r="D37" s="39">
-        <f>SE(C37&gt;12000,"Especialista",SE(C37&gt;8000,"Senior",SE(C37&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C37&gt;12000,"Especialista",IF(C37&gt;8000,"Senior",IF(C37&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E37" s="39">
-        <f>IFS(C37&gt;12000,"Especialista",C37&gt;8000,"Senior",C37&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C37&gt;12000,"Especialista",C37&gt;8000,"Senior",C37&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F37" s="40">
-        <f>SE(C37&gt;10000,"Alto",SE(C37&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C37&gt;10000,"Alto",IF(C37&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G37" s="40">
-        <f>SE(G37="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H37="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4754,19 +4754,19 @@
         <v>10781.45</v>
       </c>
       <c r="D38" s="39">
-        <f>SE(C38&gt;12000,"Especialista",SE(C38&gt;8000,"Senior",SE(C38&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C38&gt;12000,"Especialista",IF(C38&gt;8000,"Senior",IF(C38&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E38" s="39">
-        <f>IFS(C38&gt;12000,"Especialista",C38&gt;8000,"Senior",C38&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C38&gt;12000,"Especialista",C38&gt;8000,"Senior",C38&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F38" s="40">
-        <f>SE(C38&gt;10000,"Alto",SE(C38&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C38&gt;10000,"Alto",IF(C38&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G38" s="40">
-        <f>SE(G38="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H38="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4785,19 +4785,19 @@
         <v>4454.2</v>
       </c>
       <c r="D39" s="39">
-        <f>SE(C39&gt;12000,"Especialista",SE(C39&gt;8000,"Senior",SE(C39&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C39&gt;12000,"Especialista",IF(C39&gt;8000,"Senior",IF(C39&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E39" s="39">
-        <f>IFS(C39&gt;12000,"Especialista",C39&gt;8000,"Senior",C39&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C39&gt;12000,"Especialista",C39&gt;8000,"Senior",C39&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F39" s="40">
-        <f>SE(C39&gt;10000,"Alto",SE(C39&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C39&gt;10000,"Alto",IF(C39&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G39" s="40">
-        <f>SE(G39="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H39="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4816,19 +4816,19 @@
         <v>4949</v>
       </c>
       <c r="D40" s="39">
-        <f>SE(C40&gt;12000,"Especialista",SE(C40&gt;8000,"Senior",SE(C40&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C40&gt;12000,"Especialista",IF(C40&gt;8000,"Senior",IF(C40&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E40" s="39">
-        <f>IFS(C40&gt;12000,"Especialista",C40&gt;8000,"Senior",C40&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C40&gt;12000,"Especialista",C40&gt;8000,"Senior",C40&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F40" s="40">
-        <f>SE(C40&gt;10000,"Alto",SE(C40&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C40&gt;10000,"Alto",IF(C40&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G40" s="40">
-        <f>SE(G40="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H40="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4847,19 +4847,19 @@
         <v>8436.139999999999</v>
       </c>
       <c r="D41" s="39">
-        <f>SE(C41&gt;12000,"Especialista",SE(C41&gt;8000,"Senior",SE(C41&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C41&gt;12000,"Especialista",IF(C41&gt;8000,"Senior",IF(C41&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E41" s="39">
-        <f>IFS(C41&gt;12000,"Especialista",C41&gt;8000,"Senior",C41&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C41&gt;12000,"Especialista",C41&gt;8000,"Senior",C41&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F41" s="40">
-        <f>SE(C41&gt;10000,"Alto",SE(C41&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C41&gt;10000,"Alto",IF(C41&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G41" s="40">
-        <f>SE(G41="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H41="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4878,19 +4878,19 @@
         <v>4204.62</v>
       </c>
       <c r="D42" s="39">
-        <f>SE(C42&gt;12000,"Especialista",SE(C42&gt;8000,"Senior",SE(C42&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C42&gt;12000,"Especialista",IF(C42&gt;8000,"Senior",IF(C42&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E42" s="39">
-        <f>IFS(C42&gt;12000,"Especialista",C42&gt;8000,"Senior",C42&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C42&gt;12000,"Especialista",C42&gt;8000,"Senior",C42&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F42" s="40">
-        <f>SE(C42&gt;10000,"Alto",SE(C42&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C42&gt;10000,"Alto",IF(C42&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G42" s="40">
-        <f>SE(G42="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H42="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4909,19 +4909,19 @@
         <v>3399.48</v>
       </c>
       <c r="D43" s="39">
-        <f>SE(C43&gt;12000,"Especialista",SE(C43&gt;8000,"Senior",SE(C43&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C43&gt;12000,"Especialista",IF(C43&gt;8000,"Senior",IF(C43&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E43" s="39">
-        <f>IFS(C43&gt;12000,"Especialista",C43&gt;8000,"Senior",C43&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C43&gt;12000,"Especialista",C43&gt;8000,"Senior",C43&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F43" s="40">
-        <f>SE(C43&gt;10000,"Alto",SE(C43&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C43&gt;10000,"Alto",IF(C43&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G43" s="40">
-        <f>SE(G43="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H43="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4940,19 +4940,19 @@
         <v>15412.06</v>
       </c>
       <c r="D44" s="39">
-        <f>SE(C44&gt;12000,"Especialista",SE(C44&gt;8000,"Senior",SE(C44&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C44&gt;12000,"Especialista",IF(C44&gt;8000,"Senior",IF(C44&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E44" s="39">
-        <f>IFS(C44&gt;12000,"Especialista",C44&gt;8000,"Senior",C44&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C44&gt;12000,"Especialista",C44&gt;8000,"Senior",C44&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F44" s="40">
-        <f>SE(C44&gt;10000,"Alto",SE(C44&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C44&gt;10000,"Alto",IF(C44&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G44" s="40">
-        <f>SE(G44="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H44="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -4971,19 +4971,19 @@
         <v>10875.74</v>
       </c>
       <c r="D45" s="39">
-        <f>SE(C45&gt;12000,"Especialista",SE(C45&gt;8000,"Senior",SE(C45&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C45&gt;12000,"Especialista",IF(C45&gt;8000,"Senior",IF(C45&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E45" s="39">
-        <f>IFS(C45&gt;12000,"Especialista",C45&gt;8000,"Senior",C45&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C45&gt;12000,"Especialista",C45&gt;8000,"Senior",C45&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F45" s="40">
-        <f>SE(C45&gt;10000,"Alto",SE(C45&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C45&gt;10000,"Alto",IF(C45&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G45" s="40">
-        <f>SE(G45="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H45="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5002,19 +5002,19 @@
         <v>5431</v>
       </c>
       <c r="D46" s="39">
-        <f>SE(C46&gt;12000,"Especialista",SE(C46&gt;8000,"Senior",SE(C46&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C46&gt;12000,"Especialista",IF(C46&gt;8000,"Senior",IF(C46&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E46" s="39">
-        <f>IFS(C46&gt;12000,"Especialista",C46&gt;8000,"Senior",C46&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C46&gt;12000,"Especialista",C46&gt;8000,"Senior",C46&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F46" s="40">
-        <f>SE(C46&gt;10000,"Alto",SE(C46&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C46&gt;10000,"Alto",IF(C46&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G46" s="40">
-        <f>SE(G46="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H46="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5033,19 +5033,19 @@
         <v>9349.879999999999</v>
       </c>
       <c r="D47" s="39">
-        <f>SE(C47&gt;12000,"Especialista",SE(C47&gt;8000,"Senior",SE(C47&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C47&gt;12000,"Especialista",IF(C47&gt;8000,"Senior",IF(C47&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E47" s="39">
-        <f>IFS(C47&gt;12000,"Especialista",C47&gt;8000,"Senior",C47&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C47&gt;12000,"Especialista",C47&gt;8000,"Senior",C47&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F47" s="40">
-        <f>SE(C47&gt;10000,"Alto",SE(C47&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C47&gt;10000,"Alto",IF(C47&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G47" s="40">
-        <f>SE(G47="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H47="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5064,19 +5064,19 @@
         <v>5021.77</v>
       </c>
       <c r="D48" s="39">
-        <f>SE(C48&gt;12000,"Especialista",SE(C48&gt;8000,"Senior",SE(C48&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C48&gt;12000,"Especialista",IF(C48&gt;8000,"Senior",IF(C48&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E48" s="39">
-        <f>IFS(C48&gt;12000,"Especialista",C48&gt;8000,"Senior",C48&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C48&gt;12000,"Especialista",C48&gt;8000,"Senior",C48&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F48" s="40">
-        <f>SE(C48&gt;10000,"Alto",SE(C48&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C48&gt;10000,"Alto",IF(C48&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G48" s="40">
-        <f>SE(G48="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H48="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5095,19 +5095,19 @@
         <v>12760.98</v>
       </c>
       <c r="D49" s="39">
-        <f>SE(C49&gt;12000,"Especialista",SE(C49&gt;8000,"Senior",SE(C49&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C49&gt;12000,"Especialista",IF(C49&gt;8000,"Senior",IF(C49&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E49" s="39">
-        <f>IFS(C49&gt;12000,"Especialista",C49&gt;8000,"Senior",C49&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C49&gt;12000,"Especialista",C49&gt;8000,"Senior",C49&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F49" s="40">
-        <f>SE(C49&gt;10000,"Alto",SE(C49&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C49&gt;10000,"Alto",IF(C49&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G49" s="40">
-        <f>SE(G49="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H49="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5126,19 +5126,19 @@
         <v>7844.93</v>
       </c>
       <c r="D50" s="39">
-        <f>SE(C50&gt;12000,"Especialista",SE(C50&gt;8000,"Senior",SE(C50&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C50&gt;12000,"Especialista",IF(C50&gt;8000,"Senior",IF(C50&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E50" s="39">
-        <f>IFS(C50&gt;12000,"Especialista",C50&gt;8000,"Senior",C50&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C50&gt;12000,"Especialista",C50&gt;8000,"Senior",C50&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F50" s="40">
-        <f>SE(C50&gt;10000,"Alto",SE(C50&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C50&gt;10000,"Alto",IF(C50&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G50" s="40">
-        <f>SE(G50="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H50="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5157,19 +5157,19 @@
         <v>8690.25</v>
       </c>
       <c r="D51" s="39">
-        <f>SE(C51&gt;12000,"Especialista",SE(C51&gt;8000,"Senior",SE(C51&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C51&gt;12000,"Especialista",IF(C51&gt;8000,"Senior",IF(C51&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E51" s="39">
-        <f>IFS(C51&gt;12000,"Especialista",C51&gt;8000,"Senior",C51&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C51&gt;12000,"Especialista",C51&gt;8000,"Senior",C51&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F51" s="40">
-        <f>SE(C51&gt;10000,"Alto",SE(C51&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C51&gt;10000,"Alto",IF(C51&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G51" s="40">
-        <f>SE(G51="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H51="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5188,19 +5188,19 @@
         <v>7480.7</v>
       </c>
       <c r="D52" s="39">
-        <f>SE(C52&gt;12000,"Especialista",SE(C52&gt;8000,"Senior",SE(C52&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C52&gt;12000,"Especialista",IF(C52&gt;8000,"Senior",IF(C52&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E52" s="39">
-        <f>IFS(C52&gt;12000,"Especialista",C52&gt;8000,"Senior",C52&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C52&gt;12000,"Especialista",C52&gt;8000,"Senior",C52&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F52" s="40">
-        <f>SE(C52&gt;10000,"Alto",SE(C52&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C52&gt;10000,"Alto",IF(C52&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G52" s="40">
-        <f>SE(G52="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H52="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5217,19 +5217,19 @@
       </c>
       <c r="C53" s="38" t="n"/>
       <c r="D53" s="39">
-        <f>SE(C53&gt;12000,"Especialista",SE(C53&gt;8000,"Senior",SE(C53&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C53&gt;12000,"Especialista",IF(C53&gt;8000,"Senior",IF(C53&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E53" s="39">
-        <f>IFS(C53&gt;12000,"Especialista",C53&gt;8000,"Senior",C53&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C53&gt;12000,"Especialista",C53&gt;8000,"Senior",C53&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F53" s="40">
-        <f>SE(C53&gt;10000,"Alto",SE(C53&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C53&gt;10000,"Alto",IF(C53&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G53" s="40">
-        <f>SE(G53="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H53="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5248,19 +5248,19 @@
         <v>13862.23</v>
       </c>
       <c r="D54" s="39">
-        <f>SE(C54&gt;12000,"Especialista",SE(C54&gt;8000,"Senior",SE(C54&gt;5000,"Pleno","Junior")))</f>
+        <f>IF(C54&gt;12000,"Especialista",IF(C54&gt;8000,"Senior",IF(C54&gt;5000,"Pleno","Junior")))</f>
         <v/>
       </c>
       <c r="E54" s="39">
-        <f>IFS(C54&gt;12000,"Especialista",C54&gt;8000,"Senior",C54&gt;5000,"Pleno",VERDADEIRO,"Junior")</f>
+        <f>IFS(C54&gt;12000,"Especialista",C54&gt;8000,"Senior",C54&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F54" s="40">
-        <f>SE(C54&gt;10000,"Alto",SE(C54&gt;6000,"Medio","Baixo"))</f>
+        <f>IF(C54&gt;10000,"Alto",IF(C54&gt;6000,"Medio","Baixo"))</f>
         <v/>
       </c>
       <c r="G54" s="40">
-        <f>SE(G54="Sim","Ativo","Inativo")</f>
+        <f>IF(Dados!H54="Sim","Ativo","Inativo")</f>
         <v/>
       </c>
     </row>
@@ -5293,7 +5293,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>Lookup — PROCV, PROCX, INDICE+CORRESP</t>
+          <t>Lookup — VLOOKUP, XLOOKUP, INDEX+MATCH</t>
         </is>
       </c>
     </row>
@@ -5305,32 +5305,32 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>PROCV — Nome</t>
+          <t>VLOOKUP — Nome</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>PROCV — Departamento</t>
+          <t>VLOOKUP — Departamento</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>PROCV — Salario</t>
+          <t>VLOOKUP — Salario</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>PROCX — Cargo</t>
+          <t>XLOOKUP — Cargo</t>
         </is>
       </c>
       <c r="F2" s="14" t="inlineStr">
         <is>
-          <t>INDICE+CORRESP — Cidade</t>
+          <t>INDEX+MATCH — Cidade</t>
         </is>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>SEERRO — seguro</t>
+          <t>IFERROR — seguro</t>
         </is>
       </c>
     </row>
@@ -5339,27 +5339,27 @@
         <v>1</v>
       </c>
       <c r="B3" s="44">
-        <f>PROCV(A3,Dados!$A$3:$H$54,2,FALSO)</f>
+        <f>VLOOKUP(A3,Dados!$A$3:$H$54,2,FALSE)</f>
         <v/>
       </c>
       <c r="C3" s="44">
-        <f>PROCV(A3,Dados!$A$3:$H$54,3,FALSO)</f>
+        <f>VLOOKUP(A3,Dados!$A$3:$H$54,3,FALSE)</f>
         <v/>
       </c>
       <c r="D3" s="45">
-        <f>PROCV(A3,Dados!$A$3:$H$54,6,FALSO)</f>
+        <f>VLOOKUP(A3,Dados!$A$3:$H$54,6,FALSE)</f>
         <v/>
       </c>
       <c r="E3" s="46">
-        <f>PROCX(A3,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>XLOOKUP(A3,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F3" s="47">
-        <f>INDICE(Dados!$E$3:$E$54,CORRESP(A3,Dados!$A$3:$A$54,0))</f>
+        <f>INDEX(Dados!$E$3:$E$54,MATCH(A3,Dados!$A$3:$A$54,0))</f>
         <v/>
       </c>
       <c r="G3" s="48">
-        <f>SEERRO(PROCV(A3,Dados!$A$3:$H$54,2,FALSO),"ID nao encontrado")</f>
+        <f>IFERROR(VLOOKUP(A3,Dados!$A$3:$H$54,2,FALSE),"ID nao encontrado")</f>
         <v/>
       </c>
     </row>
@@ -5368,27 +5368,27 @@
         <v>5</v>
       </c>
       <c r="B4" s="44">
-        <f>PROCV(A4,Dados!$A$3:$H$54,2,FALSO)</f>
+        <f>VLOOKUP(A4,Dados!$A$3:$H$54,2,FALSE)</f>
         <v/>
       </c>
       <c r="C4" s="44">
-        <f>PROCV(A4,Dados!$A$3:$H$54,3,FALSO)</f>
+        <f>VLOOKUP(A4,Dados!$A$3:$H$54,3,FALSE)</f>
         <v/>
       </c>
       <c r="D4" s="45">
-        <f>PROCV(A4,Dados!$A$3:$H$54,6,FALSO)</f>
+        <f>VLOOKUP(A4,Dados!$A$3:$H$54,6,FALSE)</f>
         <v/>
       </c>
       <c r="E4" s="46">
-        <f>PROCX(A4,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>XLOOKUP(A4,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F4" s="47">
-        <f>INDICE(Dados!$E$3:$E$54,CORRESP(A4,Dados!$A$3:$A$54,0))</f>
+        <f>INDEX(Dados!$E$3:$E$54,MATCH(A4,Dados!$A$3:$A$54,0))</f>
         <v/>
       </c>
       <c r="G4" s="48">
-        <f>SEERRO(PROCV(A4,Dados!$A$3:$H$54,2,FALSO),"ID nao encontrado")</f>
+        <f>IFERROR(VLOOKUP(A4,Dados!$A$3:$H$54,2,FALSE),"ID nao encontrado")</f>
         <v/>
       </c>
     </row>
@@ -5397,27 +5397,27 @@
         <v>10</v>
       </c>
       <c r="B5" s="44">
-        <f>PROCV(A5,Dados!$A$3:$H$54,2,FALSO)</f>
+        <f>VLOOKUP(A5,Dados!$A$3:$H$54,2,FALSE)</f>
         <v/>
       </c>
       <c r="C5" s="44">
-        <f>PROCV(A5,Dados!$A$3:$H$54,3,FALSO)</f>
+        <f>VLOOKUP(A5,Dados!$A$3:$H$54,3,FALSE)</f>
         <v/>
       </c>
       <c r="D5" s="45">
-        <f>PROCV(A5,Dados!$A$3:$H$54,6,FALSO)</f>
+        <f>VLOOKUP(A5,Dados!$A$3:$H$54,6,FALSE)</f>
         <v/>
       </c>
       <c r="E5" s="46">
-        <f>PROCX(A5,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>XLOOKUP(A5,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F5" s="47">
-        <f>INDICE(Dados!$E$3:$E$54,CORRESP(A5,Dados!$A$3:$A$54,0))</f>
+        <f>INDEX(Dados!$E$3:$E$54,MATCH(A5,Dados!$A$3:$A$54,0))</f>
         <v/>
       </c>
       <c r="G5" s="48">
-        <f>SEERRO(PROCV(A5,Dados!$A$3:$H$54,2,FALSO),"ID nao encontrado")</f>
+        <f>IFERROR(VLOOKUP(A5,Dados!$A$3:$H$54,2,FALSE),"ID nao encontrado")</f>
         <v/>
       </c>
     </row>
@@ -5426,27 +5426,27 @@
         <v>20</v>
       </c>
       <c r="B6" s="44">
-        <f>PROCV(A6,Dados!$A$3:$H$54,2,FALSO)</f>
+        <f>VLOOKUP(A6,Dados!$A$3:$H$54,2,FALSE)</f>
         <v/>
       </c>
       <c r="C6" s="44">
-        <f>PROCV(A6,Dados!$A$3:$H$54,3,FALSO)</f>
+        <f>VLOOKUP(A6,Dados!$A$3:$H$54,3,FALSE)</f>
         <v/>
       </c>
       <c r="D6" s="45">
-        <f>PROCV(A6,Dados!$A$3:$H$54,6,FALSO)</f>
+        <f>VLOOKUP(A6,Dados!$A$3:$H$54,6,FALSE)</f>
         <v/>
       </c>
       <c r="E6" s="46">
-        <f>PROCX(A6,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>XLOOKUP(A6,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F6" s="47">
-        <f>INDICE(Dados!$E$3:$E$54,CORRESP(A6,Dados!$A$3:$A$54,0))</f>
+        <f>INDEX(Dados!$E$3:$E$54,MATCH(A6,Dados!$A$3:$A$54,0))</f>
         <v/>
       </c>
       <c r="G6" s="48">
-        <f>SEERRO(PROCV(A6,Dados!$A$3:$H$54,2,FALSO),"ID nao encontrado")</f>
+        <f>IFERROR(VLOOKUP(A6,Dados!$A$3:$H$54,2,FALSE),"ID nao encontrado")</f>
         <v/>
       </c>
     </row>
@@ -5455,27 +5455,27 @@
         <v>35</v>
       </c>
       <c r="B7" s="44">
-        <f>PROCV(A7,Dados!$A$3:$H$54,2,FALSO)</f>
+        <f>VLOOKUP(A7,Dados!$A$3:$H$54,2,FALSE)</f>
         <v/>
       </c>
       <c r="C7" s="44">
-        <f>PROCV(A7,Dados!$A$3:$H$54,3,FALSO)</f>
+        <f>VLOOKUP(A7,Dados!$A$3:$H$54,3,FALSE)</f>
         <v/>
       </c>
       <c r="D7" s="45">
-        <f>PROCV(A7,Dados!$A$3:$H$54,6,FALSO)</f>
+        <f>VLOOKUP(A7,Dados!$A$3:$H$54,6,FALSE)</f>
         <v/>
       </c>
       <c r="E7" s="46">
-        <f>PROCX(A7,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>XLOOKUP(A7,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F7" s="47">
-        <f>INDICE(Dados!$E$3:$E$54,CORRESP(A7,Dados!$A$3:$A$54,0))</f>
+        <f>INDEX(Dados!$E$3:$E$54,MATCH(A7,Dados!$A$3:$A$54,0))</f>
         <v/>
       </c>
       <c r="G7" s="48">
-        <f>SEERRO(PROCV(A7,Dados!$A$3:$H$54,2,FALSO),"ID nao encontrado")</f>
+        <f>IFERROR(VLOOKUP(A7,Dados!$A$3:$H$54,2,FALSE),"ID nao encontrado")</f>
         <v/>
       </c>
     </row>
@@ -5484,27 +5484,27 @@
         <v>50</v>
       </c>
       <c r="B8" s="44">
-        <f>PROCV(A8,Dados!$A$3:$H$54,2,FALSO)</f>
+        <f>VLOOKUP(A8,Dados!$A$3:$H$54,2,FALSE)</f>
         <v/>
       </c>
       <c r="C8" s="44">
-        <f>PROCV(A8,Dados!$A$3:$H$54,3,FALSO)</f>
+        <f>VLOOKUP(A8,Dados!$A$3:$H$54,3,FALSE)</f>
         <v/>
       </c>
       <c r="D8" s="45">
-        <f>PROCV(A8,Dados!$A$3:$H$54,6,FALSO)</f>
+        <f>VLOOKUP(A8,Dados!$A$3:$H$54,6,FALSE)</f>
         <v/>
       </c>
       <c r="E8" s="46">
-        <f>PROCX(A8,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>XLOOKUP(A8,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F8" s="47">
-        <f>INDICE(Dados!$E$3:$E$54,CORRESP(A8,Dados!$A$3:$A$54,0))</f>
+        <f>INDEX(Dados!$E$3:$E$54,MATCH(A8,Dados!$A$3:$A$54,0))</f>
         <v/>
       </c>
       <c r="G8" s="48">
-        <f>SEERRO(PROCV(A8,Dados!$A$3:$H$54,2,FALSO),"ID nao encontrado")</f>
+        <f>IFERROR(VLOOKUP(A8,Dados!$A$3:$H$54,2,FALSE),"ID nao encontrado")</f>
         <v/>
       </c>
     </row>
@@ -5513,34 +5513,34 @@
         <v>99</v>
       </c>
       <c r="B9" s="44">
-        <f>PROCV(A9,Dados!$A$3:$H$54,2,FALSO)</f>
+        <f>VLOOKUP(A9,Dados!$A$3:$H$54,2,FALSE)</f>
         <v/>
       </c>
       <c r="C9" s="44">
-        <f>PROCV(A9,Dados!$A$3:$H$54,3,FALSO)</f>
+        <f>VLOOKUP(A9,Dados!$A$3:$H$54,3,FALSE)</f>
         <v/>
       </c>
       <c r="D9" s="45">
-        <f>PROCV(A9,Dados!$A$3:$H$54,6,FALSO)</f>
+        <f>VLOOKUP(A9,Dados!$A$3:$H$54,6,FALSE)</f>
         <v/>
       </c>
       <c r="E9" s="46">
-        <f>PROCX(A9,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>XLOOKUP(A9,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F9" s="47">
-        <f>INDICE(Dados!$E$3:$E$54,CORRESP(A9,Dados!$A$3:$A$54,0))</f>
+        <f>INDEX(Dados!$E$3:$E$54,MATCH(A9,Dados!$A$3:$A$54,0))</f>
         <v/>
       </c>
       <c r="G9" s="48">
-        <f>SEERRO(PROCV(A9,Dados!$A$3:$H$54,2,FALSO),"ID nao encontrado")</f>
+        <f>IFERROR(VLOOKUP(A9,Dados!$A$3:$H$54,2,FALSE),"ID nao encontrado")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Amarelo = PROCV  |  Verde = PROCX (Excel 365+)  |  Azul = INDICE+CORRESP  |  Vermelho = SEERRO</t>
+          <t>Amarelo = VLOOKUP  |  Verde = XLOOKUP (Excel 365+)  |  Azul = INDEX+MATCH  |  Vermelho = IFERROR</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="D2" s="49" t="inlineStr">
         <is>
-          <t>Ranking (ORDEM.EQ)</t>
+          <t>Ranking (RANK.EQ)</t>
         </is>
       </c>
       <c r="F2" s="50" t="inlineStr">
@@ -5624,7 +5624,7 @@
         <v>2955.07</v>
       </c>
       <c r="D3" s="44">
-        <f>ORDEM.EQ(C3,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C3,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F3" s="15" t="inlineStr">
@@ -5633,7 +5633,7 @@
         </is>
       </c>
       <c r="G3" s="19">
-        <f>GRANDE($C$3:$C$54,1)</f>
+        <f>LARGE($C$3:$C$54,1)</f>
         <v/>
       </c>
     </row>
@@ -5648,7 +5648,7 @@
         <v>4842.67</v>
       </c>
       <c r="D4" s="44">
-        <f>ORDEM.EQ(C4,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C4,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F4" s="15" t="inlineStr">
@@ -5657,7 +5657,7 @@
         </is>
       </c>
       <c r="G4" s="19">
-        <f>GRANDE($C$3:$C$54,2)</f>
+        <f>LARGE($C$3:$C$54,2)</f>
         <v/>
       </c>
     </row>
@@ -5676,7 +5676,7 @@
         <v>8303.389999999999</v>
       </c>
       <c r="D5" s="44">
-        <f>ORDEM.EQ(C5,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C5,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -5685,7 +5685,7 @@
         </is>
       </c>
       <c r="G5" s="19">
-        <f>GRANDE($C$3:$54,3)</f>
+        <f>LARGE($C$3:$C$54,3)</f>
         <v/>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
         <v>4102.85</v>
       </c>
       <c r="D6" s="44">
-        <f>ORDEM.EQ(C6,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C6,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="G6" s="19">
-        <f>PEQUENO($C$3:$C$54,1)</f>
+        <f>SMALL($C$3:$C$54,1)</f>
         <v/>
       </c>
     </row>
@@ -5730,7 +5730,7 @@
       </c>
       <c r="C7" s="38" t="n"/>
       <c r="D7" s="44">
-        <f>ORDEM.EQ(C7,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C7,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F7" s="15" t="inlineStr">
@@ -5739,7 +5739,7 @@
         </is>
       </c>
       <c r="G7" s="19">
-        <f>MED($C$3:$C$54)</f>
+        <f>MEDIAN($C$3:$C$54)</f>
         <v/>
       </c>
     </row>
@@ -5758,7 +5758,7 @@
         <v>9059.57</v>
       </c>
       <c r="D8" s="44">
-        <f>ORDEM.EQ(C8,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C8,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F8" s="15" t="inlineStr">
@@ -5767,7 +5767,7 @@
         </is>
       </c>
       <c r="G8" s="16">
-        <f>DESVPAD($C$3:$C$54)</f>
+        <f>STDEV($C$3:$C$54)</f>
         <v/>
       </c>
     </row>
@@ -5786,7 +5786,7 @@
         <v>7459.35</v>
       </c>
       <c r="D9" s="44">
-        <f>ORDEM.EQ(C9,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C9,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F9" s="15" t="inlineStr">
@@ -5795,7 +5795,7 @@
         </is>
       </c>
       <c r="G9" s="53">
-        <f>CONT.SE($C$3:$C$54,"&gt;"&amp;MEDIA($C$3:$C$54))/CONT.VALORES($C$3:$C$54)</f>
+        <f>COUNTIF($C$3:$C$54,"&gt;"&amp;AVERAGE($C$3:$C$54))/COUNTA($C$3:$C$54)</f>
         <v/>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
       </c>
       <c r="C10" s="52" t="n"/>
       <c r="D10" s="44">
-        <f>ORDEM.EQ(C10,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C10,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F10" s="15" t="inlineStr">
@@ -5821,7 +5821,7 @@
         </is>
       </c>
       <c r="G10" s="19">
-        <f>SOMARPRODUTO(GRANDE($C$3:$C$54,{1,2,3,4,5,6,7,8,9,10}))</f>
+        <f>SUMRPRODUTO(LARGE($C$3:$C$54,{1,2,3,4,5,6,7,8,9,10}))</f>
         <v/>
       </c>
     </row>
@@ -5840,7 +5840,7 @@
         <v>4701.01</v>
       </c>
       <c r="D11" s="44">
-        <f>ORDEM.EQ(C11,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C11,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5857,7 +5857,7 @@
       </c>
       <c r="C12" s="52" t="n"/>
       <c r="D12" s="44">
-        <f>ORDEM.EQ(C12,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C12,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
         <v>7710.89</v>
       </c>
       <c r="D13" s="44">
-        <f>ORDEM.EQ(C13,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C13,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5895,7 +5895,7 @@
         <v>13862.23</v>
       </c>
       <c r="D14" s="44">
-        <f>ORDEM.EQ(C14,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C14,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5914,7 +5914,7 @@
         <v>8825.709999999999</v>
       </c>
       <c r="D15" s="44">
-        <f>ORDEM.EQ(C15,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C15,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5933,7 +5933,7 @@
         <v>9862.6</v>
       </c>
       <c r="D16" s="44">
-        <f>ORDEM.EQ(C16,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C16,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5950,7 +5950,7 @@
       </c>
       <c r="C17" s="38" t="n"/>
       <c r="D17" s="44">
-        <f>ORDEM.EQ(C17,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C17,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5969,7 +5969,7 @@
         <v>8937.76</v>
       </c>
       <c r="D18" s="44">
-        <f>ORDEM.EQ(C18,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C18,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5988,7 +5988,7 @@
         <v>7220.28</v>
       </c>
       <c r="D19" s="44">
-        <f>ORDEM.EQ(C19,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C19,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6003,7 +6003,7 @@
         <v>7324.01</v>
       </c>
       <c r="D20" s="44">
-        <f>ORDEM.EQ(C20,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C20,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6022,7 +6022,7 @@
         <v>6842.01</v>
       </c>
       <c r="D21" s="44">
-        <f>ORDEM.EQ(C21,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C21,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6041,7 +6041,7 @@
         <v>10267.47</v>
       </c>
       <c r="D22" s="44">
-        <f>ORDEM.EQ(C22,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C22,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6060,7 +6060,7 @@
         <v>3175.8</v>
       </c>
       <c r="D23" s="44">
-        <f>ORDEM.EQ(C23,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C23,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6079,7 +6079,7 @@
         <v>5123.74</v>
       </c>
       <c r="D24" s="44">
-        <f>ORDEM.EQ(C24,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C24,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6096,7 +6096,7 @@
       </c>
       <c r="C25" s="38" t="n"/>
       <c r="D25" s="44">
-        <f>ORDEM.EQ(C25,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C25,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6115,7 +6115,7 @@
         <v>9364.59</v>
       </c>
       <c r="D26" s="44">
-        <f>ORDEM.EQ(C26,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C26,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6134,7 +6134,7 @@
         <v>8983.799999999999</v>
       </c>
       <c r="D27" s="44">
-        <f>ORDEM.EQ(C27,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C27,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6153,7 +6153,7 @@
         <v>5890.78</v>
       </c>
       <c r="D28" s="44">
-        <f>ORDEM.EQ(C28,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C28,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6172,7 +6172,7 @@
         <v>10449.92</v>
       </c>
       <c r="D29" s="44">
-        <f>ORDEM.EQ(C29,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C29,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6187,7 +6187,7 @@
         <v>12224.44</v>
       </c>
       <c r="D30" s="44">
-        <f>ORDEM.EQ(C30,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C30,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6206,7 +6206,7 @@
         <v>7047.08</v>
       </c>
       <c r="D31" s="44">
-        <f>ORDEM.EQ(C31,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C31,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
         <v>6592.4</v>
       </c>
       <c r="D32" s="44">
-        <f>ORDEM.EQ(C32,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C32,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6244,7 +6244,7 @@
         <v>14651.42</v>
       </c>
       <c r="D33" s="44">
-        <f>ORDEM.EQ(C33,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C33,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
         <v>5008.97</v>
       </c>
       <c r="D34" s="44">
-        <f>ORDEM.EQ(C34,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C34,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6278,7 +6278,7 @@
         <v>8318</v>
       </c>
       <c r="D35" s="44">
-        <f>ORDEM.EQ(C35,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C35,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
         <v>9676.76</v>
       </c>
       <c r="D36" s="44">
-        <f>ORDEM.EQ(C36,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C36,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6316,7 +6316,7 @@
         <v>7730.99</v>
       </c>
       <c r="D37" s="44">
-        <f>ORDEM.EQ(C37,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C37,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
         <v>10781.45</v>
       </c>
       <c r="D38" s="44">
-        <f>ORDEM.EQ(C38,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C38,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6354,7 +6354,7 @@
         <v>4454.2</v>
       </c>
       <c r="D39" s="44">
-        <f>ORDEM.EQ(C39,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C39,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6373,7 +6373,7 @@
         <v>4949</v>
       </c>
       <c r="D40" s="44">
-        <f>ORDEM.EQ(C40,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C40,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6392,7 +6392,7 @@
         <v>8436.139999999999</v>
       </c>
       <c r="D41" s="44">
-        <f>ORDEM.EQ(C41,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C41,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6411,7 +6411,7 @@
         <v>4204.62</v>
       </c>
       <c r="D42" s="44">
-        <f>ORDEM.EQ(C42,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C42,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6430,7 +6430,7 @@
         <v>3399.48</v>
       </c>
       <c r="D43" s="44">
-        <f>ORDEM.EQ(C43,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C43,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6449,7 +6449,7 @@
         <v>15412.06</v>
       </c>
       <c r="D44" s="44">
-        <f>ORDEM.EQ(C44,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C44,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6468,7 +6468,7 @@
         <v>10875.74</v>
       </c>
       <c r="D45" s="44">
-        <f>ORDEM.EQ(C45,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C45,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
         <v>5431</v>
       </c>
       <c r="D46" s="44">
-        <f>ORDEM.EQ(C46,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C46,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6506,7 +6506,7 @@
         <v>9349.879999999999</v>
       </c>
       <c r="D47" s="44">
-        <f>ORDEM.EQ(C47,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C47,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6525,7 +6525,7 @@
         <v>5021.77</v>
       </c>
       <c r="D48" s="44">
-        <f>ORDEM.EQ(C48,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C48,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6544,7 +6544,7 @@
         <v>12760.98</v>
       </c>
       <c r="D49" s="44">
-        <f>ORDEM.EQ(C49,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C49,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6563,7 +6563,7 @@
         <v>7844.93</v>
       </c>
       <c r="D50" s="44">
-        <f>ORDEM.EQ(C50,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C50,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
         <v>8690.25</v>
       </c>
       <c r="D51" s="44">
-        <f>ORDEM.EQ(C51,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C51,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6601,7 +6601,7 @@
         <v>7480.7</v>
       </c>
       <c r="D52" s="44">
-        <f>ORDEM.EQ(C52,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C52,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6618,7 +6618,7 @@
       </c>
       <c r="C53" s="38" t="n"/>
       <c r="D53" s="44">
-        <f>ORDEM.EQ(C53,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C53,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6637,7 +6637,7 @@
         <v>13862.23</v>
       </c>
       <c r="D54" s="44">
-        <f>ORDEM.EQ(C54,$C$3:$C$54,0)</f>
+        <f>RANK.EQ(C54,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(excel): add _xlfn prefix to newer functions and remove array constants for openpyxl compatibility
</commit_message>
<xml_diff>
--- a/docs/examples/excel/cheatsheet_excel.xlsx
+++ b/docs/examples/excel/cheatsheet_excel.xlsx
@@ -2870,7 +2870,7 @@
         </is>
       </c>
       <c r="F3" s="17">
-        <f>COUNTIFS(Dados!C3:C54,"TI",Dados!H3:H54,"Sim")</f>
+        <f>COUNT_xlfn.IFS(Dados!C3:C54,"TI",Dados!H3:H54,"Sim")</f>
         <v/>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
         </is>
       </c>
       <c r="F4" s="18">
-        <f>SUMIFS(Dados!F3:F54,Dados!C3:C54,"Vendas",Dados!H3:H54,"Sim")</f>
+        <f>SUM_xlfn.IFS(Dados!F3:F54,Dados!C3:C54,"Vendas",Dados!H3:H54,"Sim")</f>
         <v/>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="F5" s="18">
-        <f>AVERAGEIFS(Dados!F3:F54,Dados!C3:C54,"TI",Dados!F3:F54,"&gt;5000")</f>
+        <f>AVERAGE_xlfn.IFS(Dados!F3:F54,Dados!C3:C54,"TI",Dados!F3:F54,"&gt;5000")</f>
         <v/>
       </c>
     </row>
@@ -3150,11 +3150,11 @@
         <v/>
       </c>
       <c r="E3" s="25">
-        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
+        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
         <v/>
       </c>
       <c r="F3" s="25">
-        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
+        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
         <v/>
       </c>
       <c r="G3" s="26">
@@ -3181,11 +3181,11 @@
         <v/>
       </c>
       <c r="E4" s="25">
-        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
+        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
         <v/>
       </c>
       <c r="F4" s="25">
-        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
+        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
         <v/>
       </c>
       <c r="G4" s="26">
@@ -3212,11 +3212,11 @@
         <v/>
       </c>
       <c r="E5" s="25">
-        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
+        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
         <v/>
       </c>
       <c r="F5" s="25">
-        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
+        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
         <v/>
       </c>
       <c r="G5" s="26">
@@ -3243,11 +3243,11 @@
         <v/>
       </c>
       <c r="E6" s="25">
-        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
+        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
         <v/>
       </c>
       <c r="F6" s="25">
-        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
+        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
         <v/>
       </c>
       <c r="G6" s="26">
@@ -3274,11 +3274,11 @@
         <v/>
       </c>
       <c r="E7" s="25">
-        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
+        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
         <v/>
       </c>
       <c r="F7" s="25">
-        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
+        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
         <v/>
       </c>
       <c r="G7" s="26">
@@ -3305,11 +3305,11 @@
         <v/>
       </c>
       <c r="E8" s="25">
-        <f>MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
+        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
         <v/>
       </c>
       <c r="F8" s="25">
-        <f>MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
+        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
         <v/>
       </c>
       <c r="G8" s="26">
@@ -3351,7 +3351,7 @@
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>Nota: MAXIFS e MINIFS requerem Excel 2019 ou 365. Em versoes mais antigas, use MAX com IFERROR(INDEX...)</t>
+          <t>Nota: _xlfn.MAXIFS e _xlfn.MINIFS requerem Excel 2019 ou 365. Em versoes mais antigas, use MAX com IFERROR(INDEX...)</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3546,7 @@
         </is>
       </c>
       <c r="F9" s="33">
-        <f>DAYS(TODAY(),Dados!G3)</f>
+        <f>_xlfn.DAYS(TODAY(),Dados!G3)</f>
         <v/>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
         <v/>
       </c>
       <c r="E3" s="39">
-        <f>IFS(C3&gt;12000,"Especialista",C3&gt;8000,"Senior",C3&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C3&gt;12000,"Especialista",C3&gt;8000,"Senior",C3&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F3" s="40">
@@ -3726,7 +3726,7 @@
         <v/>
       </c>
       <c r="E4" s="39">
-        <f>IFS(C4&gt;12000,"Especialista",C4&gt;8000,"Senior",C4&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C4&gt;12000,"Especialista",C4&gt;8000,"Senior",C4&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F4" s="40">
@@ -3757,7 +3757,7 @@
         <v/>
       </c>
       <c r="E5" s="39">
-        <f>IFS(C5&gt;12000,"Especialista",C5&gt;8000,"Senior",C5&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C5&gt;12000,"Especialista",C5&gt;8000,"Senior",C5&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F5" s="40">
@@ -3788,7 +3788,7 @@
         <v/>
       </c>
       <c r="E6" s="39">
-        <f>IFS(C6&gt;12000,"Especialista",C6&gt;8000,"Senior",C6&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C6&gt;12000,"Especialista",C6&gt;8000,"Senior",C6&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F6" s="40">
@@ -3817,7 +3817,7 @@
         <v/>
       </c>
       <c r="E7" s="39">
-        <f>IFS(C7&gt;12000,"Especialista",C7&gt;8000,"Senior",C7&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C7&gt;12000,"Especialista",C7&gt;8000,"Senior",C7&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F7" s="40">
@@ -3848,7 +3848,7 @@
         <v/>
       </c>
       <c r="E8" s="39">
-        <f>IFS(C8&gt;12000,"Especialista",C8&gt;8000,"Senior",C8&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C8&gt;12000,"Especialista",C8&gt;8000,"Senior",C8&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F8" s="40">
@@ -3879,7 +3879,7 @@
         <v/>
       </c>
       <c r="E9" s="39">
-        <f>IFS(C9&gt;12000,"Especialista",C9&gt;8000,"Senior",C9&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C9&gt;12000,"Especialista",C9&gt;8000,"Senior",C9&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F9" s="40">
@@ -3908,7 +3908,7 @@
         <v/>
       </c>
       <c r="E10" s="39">
-        <f>IFS(C10&gt;12000,"Especialista",C10&gt;8000,"Senior",C10&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C10&gt;12000,"Especialista",C10&gt;8000,"Senior",C10&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F10" s="40">
@@ -3939,7 +3939,7 @@
         <v/>
       </c>
       <c r="E11" s="39">
-        <f>IFS(C11&gt;12000,"Especialista",C11&gt;8000,"Senior",C11&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C11&gt;12000,"Especialista",C11&gt;8000,"Senior",C11&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F11" s="40">
@@ -3968,7 +3968,7 @@
         <v/>
       </c>
       <c r="E12" s="39">
-        <f>IFS(C12&gt;12000,"Especialista",C12&gt;8000,"Senior",C12&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C12&gt;12000,"Especialista",C12&gt;8000,"Senior",C12&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F12" s="40">
@@ -3999,7 +3999,7 @@
         <v/>
       </c>
       <c r="E13" s="39">
-        <f>IFS(C13&gt;12000,"Especialista",C13&gt;8000,"Senior",C13&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C13&gt;12000,"Especialista",C13&gt;8000,"Senior",C13&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F13" s="40">
@@ -4030,7 +4030,7 @@
         <v/>
       </c>
       <c r="E14" s="39">
-        <f>IFS(C14&gt;12000,"Especialista",C14&gt;8000,"Senior",C14&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C14&gt;12000,"Especialista",C14&gt;8000,"Senior",C14&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F14" s="40">
@@ -4061,7 +4061,7 @@
         <v/>
       </c>
       <c r="E15" s="39">
-        <f>IFS(C15&gt;12000,"Especialista",C15&gt;8000,"Senior",C15&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C15&gt;12000,"Especialista",C15&gt;8000,"Senior",C15&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F15" s="40">
@@ -4092,7 +4092,7 @@
         <v/>
       </c>
       <c r="E16" s="39">
-        <f>IFS(C16&gt;12000,"Especialista",C16&gt;8000,"Senior",C16&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C16&gt;12000,"Especialista",C16&gt;8000,"Senior",C16&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F16" s="40">
@@ -4121,7 +4121,7 @@
         <v/>
       </c>
       <c r="E17" s="39">
-        <f>IFS(C17&gt;12000,"Especialista",C17&gt;8000,"Senior",C17&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C17&gt;12000,"Especialista",C17&gt;8000,"Senior",C17&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F17" s="40">
@@ -4152,7 +4152,7 @@
         <v/>
       </c>
       <c r="E18" s="39">
-        <f>IFS(C18&gt;12000,"Especialista",C18&gt;8000,"Senior",C18&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C18&gt;12000,"Especialista",C18&gt;8000,"Senior",C18&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F18" s="40">
@@ -4183,7 +4183,7 @@
         <v/>
       </c>
       <c r="E19" s="39">
-        <f>IFS(C19&gt;12000,"Especialista",C19&gt;8000,"Senior",C19&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C19&gt;12000,"Especialista",C19&gt;8000,"Senior",C19&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F19" s="40">
@@ -4210,7 +4210,7 @@
         <v/>
       </c>
       <c r="E20" s="39">
-        <f>IFS(C20&gt;12000,"Especialista",C20&gt;8000,"Senior",C20&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C20&gt;12000,"Especialista",C20&gt;8000,"Senior",C20&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F20" s="40">
@@ -4241,7 +4241,7 @@
         <v/>
       </c>
       <c r="E21" s="39">
-        <f>IFS(C21&gt;12000,"Especialista",C21&gt;8000,"Senior",C21&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C21&gt;12000,"Especialista",C21&gt;8000,"Senior",C21&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F21" s="40">
@@ -4272,7 +4272,7 @@
         <v/>
       </c>
       <c r="E22" s="39">
-        <f>IFS(C22&gt;12000,"Especialista",C22&gt;8000,"Senior",C22&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C22&gt;12000,"Especialista",C22&gt;8000,"Senior",C22&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F22" s="40">
@@ -4303,7 +4303,7 @@
         <v/>
       </c>
       <c r="E23" s="39">
-        <f>IFS(C23&gt;12000,"Especialista",C23&gt;8000,"Senior",C23&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C23&gt;12000,"Especialista",C23&gt;8000,"Senior",C23&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F23" s="40">
@@ -4334,7 +4334,7 @@
         <v/>
       </c>
       <c r="E24" s="39">
-        <f>IFS(C24&gt;12000,"Especialista",C24&gt;8000,"Senior",C24&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C24&gt;12000,"Especialista",C24&gt;8000,"Senior",C24&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F24" s="40">
@@ -4363,7 +4363,7 @@
         <v/>
       </c>
       <c r="E25" s="39">
-        <f>IFS(C25&gt;12000,"Especialista",C25&gt;8000,"Senior",C25&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C25&gt;12000,"Especialista",C25&gt;8000,"Senior",C25&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F25" s="40">
@@ -4394,7 +4394,7 @@
         <v/>
       </c>
       <c r="E26" s="39">
-        <f>IFS(C26&gt;12000,"Especialista",C26&gt;8000,"Senior",C26&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C26&gt;12000,"Especialista",C26&gt;8000,"Senior",C26&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F26" s="40">
@@ -4425,7 +4425,7 @@
         <v/>
       </c>
       <c r="E27" s="39">
-        <f>IFS(C27&gt;12000,"Especialista",C27&gt;8000,"Senior",C27&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C27&gt;12000,"Especialista",C27&gt;8000,"Senior",C27&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F27" s="40">
@@ -4456,7 +4456,7 @@
         <v/>
       </c>
       <c r="E28" s="39">
-        <f>IFS(C28&gt;12000,"Especialista",C28&gt;8000,"Senior",C28&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C28&gt;12000,"Especialista",C28&gt;8000,"Senior",C28&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F28" s="40">
@@ -4487,7 +4487,7 @@
         <v/>
       </c>
       <c r="E29" s="39">
-        <f>IFS(C29&gt;12000,"Especialista",C29&gt;8000,"Senior",C29&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C29&gt;12000,"Especialista",C29&gt;8000,"Senior",C29&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F29" s="40">
@@ -4514,7 +4514,7 @@
         <v/>
       </c>
       <c r="E30" s="39">
-        <f>IFS(C30&gt;12000,"Especialista",C30&gt;8000,"Senior",C30&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C30&gt;12000,"Especialista",C30&gt;8000,"Senior",C30&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F30" s="40">
@@ -4545,7 +4545,7 @@
         <v/>
       </c>
       <c r="E31" s="39">
-        <f>IFS(C31&gt;12000,"Especialista",C31&gt;8000,"Senior",C31&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C31&gt;12000,"Especialista",C31&gt;8000,"Senior",C31&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F31" s="40">
@@ -4576,7 +4576,7 @@
         <v/>
       </c>
       <c r="E32" s="39">
-        <f>IFS(C32&gt;12000,"Especialista",C32&gt;8000,"Senior",C32&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C32&gt;12000,"Especialista",C32&gt;8000,"Senior",C32&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F32" s="40">
@@ -4607,7 +4607,7 @@
         <v/>
       </c>
       <c r="E33" s="39">
-        <f>IFS(C33&gt;12000,"Especialista",C33&gt;8000,"Senior",C33&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C33&gt;12000,"Especialista",C33&gt;8000,"Senior",C33&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F33" s="40">
@@ -4638,7 +4638,7 @@
         <v/>
       </c>
       <c r="E34" s="39">
-        <f>IFS(C34&gt;12000,"Especialista",C34&gt;8000,"Senior",C34&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C34&gt;12000,"Especialista",C34&gt;8000,"Senior",C34&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F34" s="40">
@@ -4665,7 +4665,7 @@
         <v/>
       </c>
       <c r="E35" s="39">
-        <f>IFS(C35&gt;12000,"Especialista",C35&gt;8000,"Senior",C35&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C35&gt;12000,"Especialista",C35&gt;8000,"Senior",C35&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F35" s="40">
@@ -4696,7 +4696,7 @@
         <v/>
       </c>
       <c r="E36" s="39">
-        <f>IFS(C36&gt;12000,"Especialista",C36&gt;8000,"Senior",C36&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C36&gt;12000,"Especialista",C36&gt;8000,"Senior",C36&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F36" s="40">
@@ -4727,7 +4727,7 @@
         <v/>
       </c>
       <c r="E37" s="39">
-        <f>IFS(C37&gt;12000,"Especialista",C37&gt;8000,"Senior",C37&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C37&gt;12000,"Especialista",C37&gt;8000,"Senior",C37&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F37" s="40">
@@ -4758,7 +4758,7 @@
         <v/>
       </c>
       <c r="E38" s="39">
-        <f>IFS(C38&gt;12000,"Especialista",C38&gt;8000,"Senior",C38&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C38&gt;12000,"Especialista",C38&gt;8000,"Senior",C38&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F38" s="40">
@@ -4789,7 +4789,7 @@
         <v/>
       </c>
       <c r="E39" s="39">
-        <f>IFS(C39&gt;12000,"Especialista",C39&gt;8000,"Senior",C39&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C39&gt;12000,"Especialista",C39&gt;8000,"Senior",C39&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F39" s="40">
@@ -4820,7 +4820,7 @@
         <v/>
       </c>
       <c r="E40" s="39">
-        <f>IFS(C40&gt;12000,"Especialista",C40&gt;8000,"Senior",C40&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C40&gt;12000,"Especialista",C40&gt;8000,"Senior",C40&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F40" s="40">
@@ -4851,7 +4851,7 @@
         <v/>
       </c>
       <c r="E41" s="39">
-        <f>IFS(C41&gt;12000,"Especialista",C41&gt;8000,"Senior",C41&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C41&gt;12000,"Especialista",C41&gt;8000,"Senior",C41&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F41" s="40">
@@ -4882,7 +4882,7 @@
         <v/>
       </c>
       <c r="E42" s="39">
-        <f>IFS(C42&gt;12000,"Especialista",C42&gt;8000,"Senior",C42&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C42&gt;12000,"Especialista",C42&gt;8000,"Senior",C42&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F42" s="40">
@@ -4913,7 +4913,7 @@
         <v/>
       </c>
       <c r="E43" s="39">
-        <f>IFS(C43&gt;12000,"Especialista",C43&gt;8000,"Senior",C43&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C43&gt;12000,"Especialista",C43&gt;8000,"Senior",C43&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F43" s="40">
@@ -4944,7 +4944,7 @@
         <v/>
       </c>
       <c r="E44" s="39">
-        <f>IFS(C44&gt;12000,"Especialista",C44&gt;8000,"Senior",C44&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C44&gt;12000,"Especialista",C44&gt;8000,"Senior",C44&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F44" s="40">
@@ -4975,7 +4975,7 @@
         <v/>
       </c>
       <c r="E45" s="39">
-        <f>IFS(C45&gt;12000,"Especialista",C45&gt;8000,"Senior",C45&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C45&gt;12000,"Especialista",C45&gt;8000,"Senior",C45&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F45" s="40">
@@ -5006,7 +5006,7 @@
         <v/>
       </c>
       <c r="E46" s="39">
-        <f>IFS(C46&gt;12000,"Especialista",C46&gt;8000,"Senior",C46&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C46&gt;12000,"Especialista",C46&gt;8000,"Senior",C46&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F46" s="40">
@@ -5037,7 +5037,7 @@
         <v/>
       </c>
       <c r="E47" s="39">
-        <f>IFS(C47&gt;12000,"Especialista",C47&gt;8000,"Senior",C47&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C47&gt;12000,"Especialista",C47&gt;8000,"Senior",C47&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F47" s="40">
@@ -5068,7 +5068,7 @@
         <v/>
       </c>
       <c r="E48" s="39">
-        <f>IFS(C48&gt;12000,"Especialista",C48&gt;8000,"Senior",C48&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C48&gt;12000,"Especialista",C48&gt;8000,"Senior",C48&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F48" s="40">
@@ -5099,7 +5099,7 @@
         <v/>
       </c>
       <c r="E49" s="39">
-        <f>IFS(C49&gt;12000,"Especialista",C49&gt;8000,"Senior",C49&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C49&gt;12000,"Especialista",C49&gt;8000,"Senior",C49&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F49" s="40">
@@ -5130,7 +5130,7 @@
         <v/>
       </c>
       <c r="E50" s="39">
-        <f>IFS(C50&gt;12000,"Especialista",C50&gt;8000,"Senior",C50&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C50&gt;12000,"Especialista",C50&gt;8000,"Senior",C50&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F50" s="40">
@@ -5161,7 +5161,7 @@
         <v/>
       </c>
       <c r="E51" s="39">
-        <f>IFS(C51&gt;12000,"Especialista",C51&gt;8000,"Senior",C51&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C51&gt;12000,"Especialista",C51&gt;8000,"Senior",C51&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F51" s="40">
@@ -5192,7 +5192,7 @@
         <v/>
       </c>
       <c r="E52" s="39">
-        <f>IFS(C52&gt;12000,"Especialista",C52&gt;8000,"Senior",C52&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C52&gt;12000,"Especialista",C52&gt;8000,"Senior",C52&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F52" s="40">
@@ -5221,7 +5221,7 @@
         <v/>
       </c>
       <c r="E53" s="39">
-        <f>IFS(C53&gt;12000,"Especialista",C53&gt;8000,"Senior",C53&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C53&gt;12000,"Especialista",C53&gt;8000,"Senior",C53&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F53" s="40">
@@ -5252,7 +5252,7 @@
         <v/>
       </c>
       <c r="E54" s="39">
-        <f>IFS(C54&gt;12000,"Especialista",C54&gt;8000,"Senior",C54&gt;5000,"Pleno",TRUE,"Junior")</f>
+        <f>_xlfn.IFS(C54&gt;12000,"Especialista",C54&gt;8000,"Senior",C54&gt;5000,"Pleno",TRUE,"Junior")</f>
         <v/>
       </c>
       <c r="F54" s="40">
@@ -5293,7 +5293,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>Lookup — VLOOKUP, XLOOKUP, INDEX+MATCH</t>
+          <t>Lookup — VLOOKUP, _xlfn.XLOOKUP, INDEX+MATCH</t>
         </is>
       </c>
     </row>
@@ -5320,7 +5320,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>XLOOKUP — Cargo</t>
+          <t>_xlfn.XLOOKUP — Cargo</t>
         </is>
       </c>
       <c r="F2" s="14" t="inlineStr">
@@ -5351,7 +5351,7 @@
         <v/>
       </c>
       <c r="E3" s="46">
-        <f>XLOOKUP(A3,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>_xlfn.XLOOKUP(A3,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F3" s="47">
@@ -5380,7 +5380,7 @@
         <v/>
       </c>
       <c r="E4" s="46">
-        <f>XLOOKUP(A4,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>_xlfn.XLOOKUP(A4,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F4" s="47">
@@ -5409,7 +5409,7 @@
         <v/>
       </c>
       <c r="E5" s="46">
-        <f>XLOOKUP(A5,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>_xlfn.XLOOKUP(A5,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F5" s="47">
@@ -5438,7 +5438,7 @@
         <v/>
       </c>
       <c r="E6" s="46">
-        <f>XLOOKUP(A6,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>_xlfn.XLOOKUP(A6,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F6" s="47">
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="E7" s="46">
-        <f>XLOOKUP(A7,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>_xlfn.XLOOKUP(A7,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F7" s="47">
@@ -5496,7 +5496,7 @@
         <v/>
       </c>
       <c r="E8" s="46">
-        <f>XLOOKUP(A8,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>_xlfn.XLOOKUP(A8,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F8" s="47">
@@ -5525,7 +5525,7 @@
         <v/>
       </c>
       <c r="E9" s="46">
-        <f>XLOOKUP(A9,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
+        <f>_xlfn.XLOOKUP(A9,Dados!$A$3:$A$54,Dados!$D$3:$D$54,"Nao encontrado")</f>
         <v/>
       </c>
       <c r="F9" s="47">
@@ -5540,7 +5540,7 @@
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Amarelo = VLOOKUP  |  Verde = XLOOKUP (Excel 365+)  |  Azul = INDEX+MATCH  |  Vermelho = IFERROR</t>
+          <t>Amarelo = VLOOKUP  |  Verde = _xlfn.XLOOKUP (Excel 365+)  |  Azul = INDEX+MATCH  |  Vermelho = IFERROR</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="D2" s="49" t="inlineStr">
         <is>
-          <t>Ranking (RANK.EQ)</t>
+          <t>Ranking (RANK)</t>
         </is>
       </c>
       <c r="F2" s="50" t="inlineStr">
@@ -5624,7 +5624,7 @@
         <v>2955.07</v>
       </c>
       <c r="D3" s="44">
-        <f>RANK.EQ(C3,$C$3:$C$54,0)</f>
+        <f>RANK(C3,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F3" s="15" t="inlineStr">
@@ -5648,7 +5648,7 @@
         <v>4842.67</v>
       </c>
       <c r="D4" s="44">
-        <f>RANK.EQ(C4,$C$3:$C$54,0)</f>
+        <f>RANK(C4,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F4" s="15" t="inlineStr">
@@ -5676,7 +5676,7 @@
         <v>8303.389999999999</v>
       </c>
       <c r="D5" s="44">
-        <f>RANK.EQ(C5,$C$3:$C$54,0)</f>
+        <f>RANK(C5,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -5704,7 +5704,7 @@
         <v>4102.85</v>
       </c>
       <c r="D6" s="44">
-        <f>RANK.EQ(C6,$C$3:$C$54,0)</f>
+        <f>RANK(C6,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="C7" s="38" t="n"/>
       <c r="D7" s="44">
-        <f>RANK.EQ(C7,$C$3:$C$54,0)</f>
+        <f>RANK(C7,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F7" s="15" t="inlineStr">
@@ -5758,7 +5758,7 @@
         <v>9059.57</v>
       </c>
       <c r="D8" s="44">
-        <f>RANK.EQ(C8,$C$3:$C$54,0)</f>
+        <f>RANK(C8,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F8" s="15" t="inlineStr">
@@ -5786,7 +5786,7 @@
         <v>7459.35</v>
       </c>
       <c r="D9" s="44">
-        <f>RANK.EQ(C9,$C$3:$C$54,0)</f>
+        <f>RANK(C9,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F9" s="15" t="inlineStr">
@@ -5812,12 +5812,12 @@
       </c>
       <c r="C10" s="52" t="n"/>
       <c r="D10" s="44">
-        <f>RANK.EQ(C10,$C$3:$C$54,0)</f>
+        <f>RANK(C10,$C$3:$C$54,0)</f>
         <v/>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>Folha top 10</t>
+          <t>Folha top 3</t>
         </is>
       </c>
       <c r="G10" s="19">
@@ -5840,7 +5840,7 @@
         <v>4701.01</v>
       </c>
       <c r="D11" s="44">
-        <f>RANK.EQ(C11,$C$3:$C$54,0)</f>
+        <f>RANK(C11,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5857,7 +5857,7 @@
       </c>
       <c r="C12" s="52" t="n"/>
       <c r="D12" s="44">
-        <f>RANK.EQ(C12,$C$3:$C$54,0)</f>
+        <f>RANK(C12,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
         <v>7710.89</v>
       </c>
       <c r="D13" s="44">
-        <f>RANK.EQ(C13,$C$3:$C$54,0)</f>
+        <f>RANK(C13,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5895,7 +5895,7 @@
         <v>13862.23</v>
       </c>
       <c r="D14" s="44">
-        <f>RANK.EQ(C14,$C$3:$C$54,0)</f>
+        <f>RANK(C14,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5914,7 +5914,7 @@
         <v>8825.709999999999</v>
       </c>
       <c r="D15" s="44">
-        <f>RANK.EQ(C15,$C$3:$C$54,0)</f>
+        <f>RANK(C15,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5933,7 +5933,7 @@
         <v>9862.6</v>
       </c>
       <c r="D16" s="44">
-        <f>RANK.EQ(C16,$C$3:$C$54,0)</f>
+        <f>RANK(C16,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5950,7 +5950,7 @@
       </c>
       <c r="C17" s="38" t="n"/>
       <c r="D17" s="44">
-        <f>RANK.EQ(C17,$C$3:$C$54,0)</f>
+        <f>RANK(C17,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5969,7 +5969,7 @@
         <v>8937.76</v>
       </c>
       <c r="D18" s="44">
-        <f>RANK.EQ(C18,$C$3:$C$54,0)</f>
+        <f>RANK(C18,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -5988,7 +5988,7 @@
         <v>7220.28</v>
       </c>
       <c r="D19" s="44">
-        <f>RANK.EQ(C19,$C$3:$C$54,0)</f>
+        <f>RANK(C19,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6003,7 +6003,7 @@
         <v>7324.01</v>
       </c>
       <c r="D20" s="44">
-        <f>RANK.EQ(C20,$C$3:$C$54,0)</f>
+        <f>RANK(C20,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6022,7 +6022,7 @@
         <v>6842.01</v>
       </c>
       <c r="D21" s="44">
-        <f>RANK.EQ(C21,$C$3:$C$54,0)</f>
+        <f>RANK(C21,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6041,7 +6041,7 @@
         <v>10267.47</v>
       </c>
       <c r="D22" s="44">
-        <f>RANK.EQ(C22,$C$3:$C$54,0)</f>
+        <f>RANK(C22,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6060,7 +6060,7 @@
         <v>3175.8</v>
       </c>
       <c r="D23" s="44">
-        <f>RANK.EQ(C23,$C$3:$C$54,0)</f>
+        <f>RANK(C23,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6079,7 +6079,7 @@
         <v>5123.74</v>
       </c>
       <c r="D24" s="44">
-        <f>RANK.EQ(C24,$C$3:$C$54,0)</f>
+        <f>RANK(C24,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6096,7 +6096,7 @@
       </c>
       <c r="C25" s="38" t="n"/>
       <c r="D25" s="44">
-        <f>RANK.EQ(C25,$C$3:$C$54,0)</f>
+        <f>RANK(C25,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6115,7 +6115,7 @@
         <v>9364.59</v>
       </c>
       <c r="D26" s="44">
-        <f>RANK.EQ(C26,$C$3:$C$54,0)</f>
+        <f>RANK(C26,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6134,7 +6134,7 @@
         <v>8983.799999999999</v>
       </c>
       <c r="D27" s="44">
-        <f>RANK.EQ(C27,$C$3:$C$54,0)</f>
+        <f>RANK(C27,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6153,7 +6153,7 @@
         <v>5890.78</v>
       </c>
       <c r="D28" s="44">
-        <f>RANK.EQ(C28,$C$3:$C$54,0)</f>
+        <f>RANK(C28,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6172,7 +6172,7 @@
         <v>10449.92</v>
       </c>
       <c r="D29" s="44">
-        <f>RANK.EQ(C29,$C$3:$C$54,0)</f>
+        <f>RANK(C29,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6187,7 +6187,7 @@
         <v>12224.44</v>
       </c>
       <c r="D30" s="44">
-        <f>RANK.EQ(C30,$C$3:$C$54,0)</f>
+        <f>RANK(C30,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6206,7 +6206,7 @@
         <v>7047.08</v>
       </c>
       <c r="D31" s="44">
-        <f>RANK.EQ(C31,$C$3:$C$54,0)</f>
+        <f>RANK(C31,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
         <v>6592.4</v>
       </c>
       <c r="D32" s="44">
-        <f>RANK.EQ(C32,$C$3:$C$54,0)</f>
+        <f>RANK(C32,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6244,7 +6244,7 @@
         <v>14651.42</v>
       </c>
       <c r="D33" s="44">
-        <f>RANK.EQ(C33,$C$3:$C$54,0)</f>
+        <f>RANK(C33,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
         <v>5008.97</v>
       </c>
       <c r="D34" s="44">
-        <f>RANK.EQ(C34,$C$3:$C$54,0)</f>
+        <f>RANK(C34,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6278,7 +6278,7 @@
         <v>8318</v>
       </c>
       <c r="D35" s="44">
-        <f>RANK.EQ(C35,$C$3:$C$54,0)</f>
+        <f>RANK(C35,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
         <v>9676.76</v>
       </c>
       <c r="D36" s="44">
-        <f>RANK.EQ(C36,$C$3:$C$54,0)</f>
+        <f>RANK(C36,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6316,7 +6316,7 @@
         <v>7730.99</v>
       </c>
       <c r="D37" s="44">
-        <f>RANK.EQ(C37,$C$3:$C$54,0)</f>
+        <f>RANK(C37,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
         <v>10781.45</v>
       </c>
       <c r="D38" s="44">
-        <f>RANK.EQ(C38,$C$3:$C$54,0)</f>
+        <f>RANK(C38,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6354,7 +6354,7 @@
         <v>4454.2</v>
       </c>
       <c r="D39" s="44">
-        <f>RANK.EQ(C39,$C$3:$C$54,0)</f>
+        <f>RANK(C39,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6373,7 +6373,7 @@
         <v>4949</v>
       </c>
       <c r="D40" s="44">
-        <f>RANK.EQ(C40,$C$3:$C$54,0)</f>
+        <f>RANK(C40,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6392,7 +6392,7 @@
         <v>8436.139999999999</v>
       </c>
       <c r="D41" s="44">
-        <f>RANK.EQ(C41,$C$3:$C$54,0)</f>
+        <f>RANK(C41,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6411,7 +6411,7 @@
         <v>4204.62</v>
       </c>
       <c r="D42" s="44">
-        <f>RANK.EQ(C42,$C$3:$C$54,0)</f>
+        <f>RANK(C42,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6430,7 +6430,7 @@
         <v>3399.48</v>
       </c>
       <c r="D43" s="44">
-        <f>RANK.EQ(C43,$C$3:$C$54,0)</f>
+        <f>RANK(C43,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6449,7 +6449,7 @@
         <v>15412.06</v>
       </c>
       <c r="D44" s="44">
-        <f>RANK.EQ(C44,$C$3:$C$54,0)</f>
+        <f>RANK(C44,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6468,7 +6468,7 @@
         <v>10875.74</v>
       </c>
       <c r="D45" s="44">
-        <f>RANK.EQ(C45,$C$3:$C$54,0)</f>
+        <f>RANK(C45,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
         <v>5431</v>
       </c>
       <c r="D46" s="44">
-        <f>RANK.EQ(C46,$C$3:$C$54,0)</f>
+        <f>RANK(C46,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6506,7 +6506,7 @@
         <v>9349.879999999999</v>
       </c>
       <c r="D47" s="44">
-        <f>RANK.EQ(C47,$C$3:$C$54,0)</f>
+        <f>RANK(C47,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6525,7 +6525,7 @@
         <v>5021.77</v>
       </c>
       <c r="D48" s="44">
-        <f>RANK.EQ(C48,$C$3:$C$54,0)</f>
+        <f>RANK(C48,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6544,7 +6544,7 @@
         <v>12760.98</v>
       </c>
       <c r="D49" s="44">
-        <f>RANK.EQ(C49,$C$3:$C$54,0)</f>
+        <f>RANK(C49,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6563,7 +6563,7 @@
         <v>7844.93</v>
       </c>
       <c r="D50" s="44">
-        <f>RANK.EQ(C50,$C$3:$C$54,0)</f>
+        <f>RANK(C50,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
         <v>8690.25</v>
       </c>
       <c r="D51" s="44">
-        <f>RANK.EQ(C51,$C$3:$C$54,0)</f>
+        <f>RANK(C51,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6601,7 +6601,7 @@
         <v>7480.7</v>
       </c>
       <c r="D52" s="44">
-        <f>RANK.EQ(C52,$C$3:$C$54,0)</f>
+        <f>RANK(C52,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6618,7 +6618,7 @@
       </c>
       <c r="C53" s="38" t="n"/>
       <c r="D53" s="44">
-        <f>RANK.EQ(C53,$C$3:$C$54,0)</f>
+        <f>RANK(C53,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>
@@ -6637,7 +6637,7 @@
         <v>13862.23</v>
       </c>
       <c r="D54" s="44">
-        <f>RANK.EQ(C54,$C$3:$C$54,0)</f>
+        <f>RANK(C54,$C$3:$C$54,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(excel): resolve substring replacement bug that corrupted COUNTIFS, SUMIFS, MAXIFS and MINIFS formulas
</commit_message>
<xml_diff>
--- a/docs/examples/excel/cheatsheet_excel.xlsx
+++ b/docs/examples/excel/cheatsheet_excel.xlsx
@@ -2870,7 +2870,7 @@
         </is>
       </c>
       <c r="F3" s="17">
-        <f>COUNT_xlfn.IFS(Dados!C3:C54,"TI",Dados!H3:H54,"Sim")</f>
+        <f>COUNTIFS(Dados!C3:C54,"TI",Dados!H3:H54,"Sim")</f>
         <v/>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
         </is>
       </c>
       <c r="F4" s="18">
-        <f>SUM_xlfn.IFS(Dados!F3:F54,Dados!C3:C54,"Vendas",Dados!H3:H54,"Sim")</f>
+        <f>SUMIFS(Dados!F3:F54,Dados!C3:C54,"Vendas",Dados!H3:H54,"Sim")</f>
         <v/>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="F5" s="18">
-        <f>AVERAGE_xlfn.IFS(Dados!F3:F54,Dados!C3:C54,"TI",Dados!F3:F54,"&gt;5000")</f>
+        <f>AVERAGEIFS(Dados!F3:F54,Dados!C3:C54,"TI",Dados!F3:F54,"&gt;5000")</f>
         <v/>
       </c>
     </row>
@@ -3150,11 +3150,11 @@
         <v/>
       </c>
       <c r="E3" s="25">
-        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
+        <f>_xlfn.MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
         <v/>
       </c>
       <c r="F3" s="25">
-        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
+        <f>_xlfn.MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A3)</f>
         <v/>
       </c>
       <c r="G3" s="26">
@@ -3181,11 +3181,11 @@
         <v/>
       </c>
       <c r="E4" s="25">
-        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
+        <f>_xlfn.MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
         <v/>
       </c>
       <c r="F4" s="25">
-        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
+        <f>_xlfn.MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A4)</f>
         <v/>
       </c>
       <c r="G4" s="26">
@@ -3212,11 +3212,11 @@
         <v/>
       </c>
       <c r="E5" s="25">
-        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
+        <f>_xlfn.MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
         <v/>
       </c>
       <c r="F5" s="25">
-        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
+        <f>_xlfn.MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A5)</f>
         <v/>
       </c>
       <c r="G5" s="26">
@@ -3243,11 +3243,11 @@
         <v/>
       </c>
       <c r="E6" s="25">
-        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
+        <f>_xlfn.MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
         <v/>
       </c>
       <c r="F6" s="25">
-        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
+        <f>_xlfn.MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A6)</f>
         <v/>
       </c>
       <c r="G6" s="26">
@@ -3274,11 +3274,11 @@
         <v/>
       </c>
       <c r="E7" s="25">
-        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
+        <f>_xlfn.MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
         <v/>
       </c>
       <c r="F7" s="25">
-        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
+        <f>_xlfn.MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A7)</f>
         <v/>
       </c>
       <c r="G7" s="26">
@@ -3305,11 +3305,11 @@
         <v/>
       </c>
       <c r="E8" s="25">
-        <f>MAX_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
+        <f>_xlfn.MAXIFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
         <v/>
       </c>
       <c r="F8" s="25">
-        <f>MIN_xlfn.IFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
+        <f>_xlfn.MINIFS(Dados!F$3:F$54,Dados!C$3:C$54,A8)</f>
         <v/>
       </c>
       <c r="G8" s="26">

</xml_diff>

<commit_message>
fix(excel): resolve formula logic bugs, missing formats, div/0 and text IDs
</commit_message>
<xml_diff>
--- a/docs/examples/excel/cheatsheet_excel.xlsx
+++ b/docs/examples/excel/cheatsheet_excel.xlsx
@@ -244,8 +244,8 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -709,10 +709,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A3" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -758,10 +756,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A4" s="9" t="n">
+        <v>2</v>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
@@ -803,10 +799,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="A5" s="4" t="n">
+        <v>3</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -852,10 +846,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="A6" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
@@ -901,10 +893,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="A7" s="4" t="n">
+        <v>5</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -948,10 +938,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="A8" s="9" t="n">
+        <v>6</v>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
@@ -997,10 +985,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="A9" s="4" t="n">
+        <v>7</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -1046,10 +1032,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="A10" s="9" t="n">
+        <v>8</v>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
@@ -1084,10 +1068,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
+      <c r="A11" s="4" t="n">
+        <v>9</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
@@ -1124,10 +1106,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="A12" s="9" t="n">
+        <v>10</v>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
@@ -1162,10 +1142,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="A13" s="4" t="n">
+        <v>11</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
@@ -1202,10 +1180,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="A14" s="9" t="n">
+        <v>12</v>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
@@ -1242,10 +1218,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="A15" s="4" t="n">
+        <v>13</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -1282,10 +1256,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="A16" s="9" t="n">
+        <v>14</v>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
@@ -1322,10 +1294,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="A17" s="4" t="n">
+        <v>15</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
@@ -1360,10 +1330,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="A18" s="9" t="n">
+        <v>16</v>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
@@ -1400,10 +1368,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
+      <c r="A19" s="4" t="n">
+        <v>17</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
@@ -1440,10 +1406,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="A20" s="9" t="n">
+        <v>18</v>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
@@ -1476,10 +1440,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
+      <c r="A21" s="4" t="n">
+        <v>19</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
@@ -1516,10 +1478,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="A22" s="9" t="n">
+        <v>20</v>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
@@ -1552,10 +1512,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
+      <c r="A23" s="4" t="n">
+        <v>21</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
@@ -1592,10 +1550,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+      <c r="A24" s="9" t="n">
+        <v>22</v>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
@@ -1628,10 +1584,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+      <c r="A25" s="4" t="n">
+        <v>23</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
@@ -1666,10 +1620,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="A26" s="9" t="n">
+        <v>24</v>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
@@ -1706,10 +1658,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
+      <c r="A27" s="4" t="n">
+        <v>25</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
@@ -1746,10 +1696,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
+      <c r="A28" s="9" t="n">
+        <v>26</v>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
@@ -1786,10 +1734,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
+      <c r="A29" s="4" t="n">
+        <v>27</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
@@ -1826,10 +1772,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+      <c r="A30" s="9" t="n">
+        <v>28</v>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
@@ -1862,10 +1806,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="A31" s="4" t="n">
+        <v>29</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
@@ -1902,10 +1844,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="A32" s="9" t="n">
+        <v>30</v>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
@@ -1942,10 +1882,8 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="A33" s="4" t="n">
+        <v>31</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
@@ -1982,10 +1920,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
+      <c r="A34" s="9" t="n">
+        <v>32</v>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
@@ -2018,10 +1954,8 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="A35" s="4" t="n">
+        <v>33</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
@@ -2050,10 +1984,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
+      <c r="A36" s="9" t="n">
+        <v>34</v>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
@@ -2090,10 +2022,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="A37" s="4" t="n">
+        <v>35</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
@@ -2130,10 +2060,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
+      <c r="A38" s="9" t="n">
+        <v>36</v>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
@@ -2170,10 +2098,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="A39" s="4" t="n">
+        <v>37</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
@@ -2210,10 +2136,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
+      <c r="A40" s="9" t="n">
+        <v>38</v>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
@@ -2246,10 +2170,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
+      <c r="A41" s="4" t="n">
+        <v>39</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
@@ -2286,10 +2208,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
+      <c r="A42" s="9" t="n">
+        <v>40</v>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
@@ -2326,10 +2246,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
+      <c r="A43" s="4" t="n">
+        <v>41</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
@@ -2366,10 +2284,8 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
+      <c r="A44" s="9" t="n">
+        <v>42</v>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
@@ -2406,10 +2322,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
+      <c r="A45" s="4" t="n">
+        <v>43</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
@@ -2446,10 +2360,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
+      <c r="A46" s="9" t="n">
+        <v>44</v>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
@@ -2486,10 +2398,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="A47" s="4" t="n">
+        <v>45</v>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
@@ -2526,10 +2436,8 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
+      <c r="A48" s="9" t="n">
+        <v>46</v>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
@@ -2562,10 +2470,8 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
+      <c r="A49" s="4" t="n">
+        <v>47</v>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
@@ -2602,10 +2508,8 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
+      <c r="A50" s="9" t="n">
+        <v>48</v>
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
@@ -2642,10 +2546,8 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
+      <c r="A51" s="4" t="n">
+        <v>49</v>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
@@ -2682,10 +2584,8 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="A52" s="9" t="n">
+        <v>50</v>
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
@@ -2722,10 +2622,8 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
+      <c r="A53" s="4" t="n">
+        <v>51</v>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
@@ -2760,10 +2658,8 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="9" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
+      <c r="A54" s="9" t="n">
+        <v>52</v>
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
@@ -3010,7 +2906,7 @@
         </is>
       </c>
       <c r="F10" s="18">
-        <f>SUMRPRODUTO(1/COUNTIF(Dados!C3:C53,Dados!C3:C53))</f>
+        <f>SUMPRODUCT(1/COUNTIF(Dados!C3:C53,Dados!C3:C53))</f>
         <v/>
       </c>
     </row>
@@ -3146,7 +3042,7 @@
         <v/>
       </c>
       <c r="D3" s="25">
-        <f>AVERAGEIF(Dados!C$3:C$54,A3,Dados!F$3:F$54)</f>
+        <f>IFERROR(AVERAGEIF(Dados!C$3:C$54,A3,Dados!F$3:F$54),0)</f>
         <v/>
       </c>
       <c r="E3" s="25">
@@ -3177,7 +3073,7 @@
         <v/>
       </c>
       <c r="D4" s="25">
-        <f>AVERAGEIF(Dados!C$3:C$54,A4,Dados!F$3:F$54)</f>
+        <f>IFERROR(AVERAGEIF(Dados!C$3:C$54,A4,Dados!F$3:F$54),0)</f>
         <v/>
       </c>
       <c r="E4" s="25">
@@ -3208,7 +3104,7 @@
         <v/>
       </c>
       <c r="D5" s="25">
-        <f>AVERAGEIF(Dados!C$3:C$54,A5,Dados!F$3:F$54)</f>
+        <f>IFERROR(AVERAGEIF(Dados!C$3:C$54,A5,Dados!F$3:F$54),0)</f>
         <v/>
       </c>
       <c r="E5" s="25">
@@ -3239,7 +3135,7 @@
         <v/>
       </c>
       <c r="D6" s="25">
-        <f>AVERAGEIF(Dados!C$3:C$54,A6,Dados!F$3:F$54)</f>
+        <f>IFERROR(AVERAGEIF(Dados!C$3:C$54,A6,Dados!F$3:F$54),0)</f>
         <v/>
       </c>
       <c r="E6" s="25">
@@ -3270,7 +3166,7 @@
         <v/>
       </c>
       <c r="D7" s="25">
-        <f>AVERAGEIF(Dados!C$3:C$54,A7,Dados!F$3:F$54)</f>
+        <f>IFERROR(AVERAGEIF(Dados!C$3:C$54,A7,Dados!F$3:F$54),0)</f>
         <v/>
       </c>
       <c r="E7" s="25">
@@ -3301,7 +3197,7 @@
         <v/>
       </c>
       <c r="D8" s="25">
-        <f>AVERAGEIF(Dados!C$3:C$54,A8,Dados!F$3:F$54)</f>
+        <f>IFERROR(AVERAGEIF(Dados!C$3:C$54,A8,Dados!F$3:F$54),0)</f>
         <v/>
       </c>
       <c r="E8" s="25">
@@ -3425,7 +3321,7 @@
           <t>Tempo de casa (dias)</t>
         </is>
       </c>
-      <c r="F3" s="17">
+      <c r="F3" s="32">
         <f>TODAY()-Dados!G3</f>
         <v/>
       </c>
@@ -3445,8 +3341,8 @@
           <t>Tempo de casa (anos)</t>
         </is>
       </c>
-      <c r="F4" s="32">
-        <f>FRAÇÃO.YEAR(Dados!G3,TODAY())</f>
+      <c r="F4" s="33">
+        <f>YEARFRAC(Dados!G3,TODAY())</f>
         <v/>
       </c>
     </row>
@@ -3466,7 +3362,7 @@
         </is>
       </c>
       <c r="F5" s="17">
-        <f>EDATE(Dados!G3,0)</f>
+        <f>DATEDIF(Dados!G3,TODAY(),"M")</f>
         <v/>
       </c>
     </row>
@@ -3485,7 +3381,7 @@
           <t>Data + 30 dias</t>
         </is>
       </c>
-      <c r="F6" s="33">
+      <c r="F6" s="32">
         <f>Dados!G3+30</f>
         <v/>
       </c>
@@ -3505,7 +3401,7 @@
           <t>Primeiro dia do mes</t>
         </is>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="32">
         <f>DATE(YEAR(Dados!G3),MONTH(Dados!G3),1)</f>
         <v/>
       </c>
@@ -3525,7 +3421,7 @@
           <t>Ultimo dia do mes</t>
         </is>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="32">
         <f>EOMONTH(Dados!G3,0)</f>
         <v/>
       </c>
@@ -3545,7 +3441,7 @@
           <t>Dias entre duas datas</t>
         </is>
       </c>
-      <c r="F9" s="33">
+      <c r="F9" s="32">
         <f>_xlfn.DAYS(TODAY(),Dados!G3)</f>
         <v/>
       </c>
@@ -3565,7 +3461,7 @@
           <t>Dias uteis entre datas</t>
         </is>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="32">
         <f>WORKDAY(Dados!G3,30)</f>
         <v/>
       </c>
@@ -3605,7 +3501,7 @@
           <t>Mais recente admissao</t>
         </is>
       </c>
-      <c r="F12" s="33">
+      <c r="F12" s="32">
         <f>MAX(Dados!G3:G54)</f>
         <v/>
       </c>
@@ -5624,7 +5520,7 @@
         <v>2955.07</v>
       </c>
       <c r="D3" s="44">
-        <f>RANK(C3,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C3), "", RANK(C3,$C$3:$C$54,0))</f>
         <v/>
       </c>
       <c r="F3" s="15" t="inlineStr">
@@ -5648,7 +5544,7 @@
         <v>4842.67</v>
       </c>
       <c r="D4" s="44">
-        <f>RANK(C4,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C4), "", RANK(C4,$C$3:$C$54,0))</f>
         <v/>
       </c>
       <c r="F4" s="15" t="inlineStr">
@@ -5676,7 +5572,7 @@
         <v>8303.389999999999</v>
       </c>
       <c r="D5" s="44">
-        <f>RANK(C5,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C5), "", RANK(C5,$C$3:$C$54,0))</f>
         <v/>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -5704,7 +5600,7 @@
         <v>4102.85</v>
       </c>
       <c r="D6" s="44">
-        <f>RANK(C6,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C6), "", RANK(C6,$C$3:$C$54,0))</f>
         <v/>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -5730,7 +5626,7 @@
       </c>
       <c r="C7" s="38" t="n"/>
       <c r="D7" s="44">
-        <f>RANK(C7,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C7), "", RANK(C7,$C$3:$C$54,0))</f>
         <v/>
       </c>
       <c r="F7" s="15" t="inlineStr">
@@ -5758,7 +5654,7 @@
         <v>9059.57</v>
       </c>
       <c r="D8" s="44">
-        <f>RANK(C8,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C8), "", RANK(C8,$C$3:$C$54,0))</f>
         <v/>
       </c>
       <c r="F8" s="15" t="inlineStr">
@@ -5786,7 +5682,7 @@
         <v>7459.35</v>
       </c>
       <c r="D9" s="44">
-        <f>RANK(C9,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C9), "", RANK(C9,$C$3:$C$54,0))</f>
         <v/>
       </c>
       <c r="F9" s="15" t="inlineStr">
@@ -5812,7 +5708,7 @@
       </c>
       <c r="C10" s="52" t="n"/>
       <c r="D10" s="44">
-        <f>RANK(C10,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C10), "", RANK(C10,$C$3:$C$54,0))</f>
         <v/>
       </c>
       <c r="F10" s="15" t="inlineStr">
@@ -5821,7 +5717,7 @@
         </is>
       </c>
       <c r="G10" s="19">
-        <f>SUMRPRODUTO(LARGE($C$3:$C$54,{1,2,3,4,5,6,7,8,9,10}))</f>
+        <f>LARGE($C$3:$C$54,1)+LARGE($C$3:$C$54,2)+LARGE($C$3:$C$54,3)</f>
         <v/>
       </c>
     </row>
@@ -5840,7 +5736,7 @@
         <v>4701.01</v>
       </c>
       <c r="D11" s="44">
-        <f>RANK(C11,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C11), "", RANK(C11,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -5857,7 +5753,7 @@
       </c>
       <c r="C12" s="52" t="n"/>
       <c r="D12" s="44">
-        <f>RANK(C12,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C12), "", RANK(C12,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -5876,7 +5772,7 @@
         <v>7710.89</v>
       </c>
       <c r="D13" s="44">
-        <f>RANK(C13,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C13), "", RANK(C13,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -5895,7 +5791,7 @@
         <v>13862.23</v>
       </c>
       <c r="D14" s="44">
-        <f>RANK(C14,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C14), "", RANK(C14,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -5914,7 +5810,7 @@
         <v>8825.709999999999</v>
       </c>
       <c r="D15" s="44">
-        <f>RANK(C15,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C15), "", RANK(C15,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -5933,7 +5829,7 @@
         <v>9862.6</v>
       </c>
       <c r="D16" s="44">
-        <f>RANK(C16,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C16), "", RANK(C16,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -5950,7 +5846,7 @@
       </c>
       <c r="C17" s="38" t="n"/>
       <c r="D17" s="44">
-        <f>RANK(C17,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C17), "", RANK(C17,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -5969,7 +5865,7 @@
         <v>8937.76</v>
       </c>
       <c r="D18" s="44">
-        <f>RANK(C18,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C18), "", RANK(C18,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -5988,7 +5884,7 @@
         <v>7220.28</v>
       </c>
       <c r="D19" s="44">
-        <f>RANK(C19,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C19), "", RANK(C19,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6003,7 +5899,7 @@
         <v>7324.01</v>
       </c>
       <c r="D20" s="44">
-        <f>RANK(C20,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C20), "", RANK(C20,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6022,7 +5918,7 @@
         <v>6842.01</v>
       </c>
       <c r="D21" s="44">
-        <f>RANK(C21,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C21), "", RANK(C21,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6041,7 +5937,7 @@
         <v>10267.47</v>
       </c>
       <c r="D22" s="44">
-        <f>RANK(C22,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C22), "", RANK(C22,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6060,7 +5956,7 @@
         <v>3175.8</v>
       </c>
       <c r="D23" s="44">
-        <f>RANK(C23,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C23), "", RANK(C23,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6079,7 +5975,7 @@
         <v>5123.74</v>
       </c>
       <c r="D24" s="44">
-        <f>RANK(C24,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C24), "", RANK(C24,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6096,7 +5992,7 @@
       </c>
       <c r="C25" s="38" t="n"/>
       <c r="D25" s="44">
-        <f>RANK(C25,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C25), "", RANK(C25,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6115,7 +6011,7 @@
         <v>9364.59</v>
       </c>
       <c r="D26" s="44">
-        <f>RANK(C26,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C26), "", RANK(C26,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6134,7 +6030,7 @@
         <v>8983.799999999999</v>
       </c>
       <c r="D27" s="44">
-        <f>RANK(C27,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C27), "", RANK(C27,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6153,7 +6049,7 @@
         <v>5890.78</v>
       </c>
       <c r="D28" s="44">
-        <f>RANK(C28,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C28), "", RANK(C28,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6172,7 +6068,7 @@
         <v>10449.92</v>
       </c>
       <c r="D29" s="44">
-        <f>RANK(C29,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C29), "", RANK(C29,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6187,7 +6083,7 @@
         <v>12224.44</v>
       </c>
       <c r="D30" s="44">
-        <f>RANK(C30,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C30), "", RANK(C30,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6206,7 +6102,7 @@
         <v>7047.08</v>
       </c>
       <c r="D31" s="44">
-        <f>RANK(C31,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C31), "", RANK(C31,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6225,7 +6121,7 @@
         <v>6592.4</v>
       </c>
       <c r="D32" s="44">
-        <f>RANK(C32,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C32), "", RANK(C32,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6244,7 +6140,7 @@
         <v>14651.42</v>
       </c>
       <c r="D33" s="44">
-        <f>RANK(C33,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C33), "", RANK(C33,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6263,7 +6159,7 @@
         <v>5008.97</v>
       </c>
       <c r="D34" s="44">
-        <f>RANK(C34,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C34), "", RANK(C34,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6278,7 +6174,7 @@
         <v>8318</v>
       </c>
       <c r="D35" s="44">
-        <f>RANK(C35,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C35), "", RANK(C35,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6297,7 +6193,7 @@
         <v>9676.76</v>
       </c>
       <c r="D36" s="44">
-        <f>RANK(C36,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C36), "", RANK(C36,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6316,7 +6212,7 @@
         <v>7730.99</v>
       </c>
       <c r="D37" s="44">
-        <f>RANK(C37,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C37), "", RANK(C37,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6335,7 +6231,7 @@
         <v>10781.45</v>
       </c>
       <c r="D38" s="44">
-        <f>RANK(C38,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C38), "", RANK(C38,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6354,7 +6250,7 @@
         <v>4454.2</v>
       </c>
       <c r="D39" s="44">
-        <f>RANK(C39,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C39), "", RANK(C39,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6373,7 +6269,7 @@
         <v>4949</v>
       </c>
       <c r="D40" s="44">
-        <f>RANK(C40,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C40), "", RANK(C40,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6392,7 +6288,7 @@
         <v>8436.139999999999</v>
       </c>
       <c r="D41" s="44">
-        <f>RANK(C41,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C41), "", RANK(C41,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6411,7 +6307,7 @@
         <v>4204.62</v>
       </c>
       <c r="D42" s="44">
-        <f>RANK(C42,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C42), "", RANK(C42,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6430,7 +6326,7 @@
         <v>3399.48</v>
       </c>
       <c r="D43" s="44">
-        <f>RANK(C43,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C43), "", RANK(C43,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6449,7 +6345,7 @@
         <v>15412.06</v>
       </c>
       <c r="D44" s="44">
-        <f>RANK(C44,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C44), "", RANK(C44,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6468,7 +6364,7 @@
         <v>10875.74</v>
       </c>
       <c r="D45" s="44">
-        <f>RANK(C45,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C45), "", RANK(C45,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6487,7 +6383,7 @@
         <v>5431</v>
       </c>
       <c r="D46" s="44">
-        <f>RANK(C46,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C46), "", RANK(C46,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6506,7 +6402,7 @@
         <v>9349.879999999999</v>
       </c>
       <c r="D47" s="44">
-        <f>RANK(C47,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C47), "", RANK(C47,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6525,7 +6421,7 @@
         <v>5021.77</v>
       </c>
       <c r="D48" s="44">
-        <f>RANK(C48,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C48), "", RANK(C48,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6544,7 +6440,7 @@
         <v>12760.98</v>
       </c>
       <c r="D49" s="44">
-        <f>RANK(C49,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C49), "", RANK(C49,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6563,7 +6459,7 @@
         <v>7844.93</v>
       </c>
       <c r="D50" s="44">
-        <f>RANK(C50,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C50), "", RANK(C50,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6582,7 +6478,7 @@
         <v>8690.25</v>
       </c>
       <c r="D51" s="44">
-        <f>RANK(C51,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C51), "", RANK(C51,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6601,7 +6497,7 @@
         <v>7480.7</v>
       </c>
       <c r="D52" s="44">
-        <f>RANK(C52,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C52), "", RANK(C52,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6618,7 +6514,7 @@
       </c>
       <c r="C53" s="38" t="n"/>
       <c r="D53" s="44">
-        <f>RANK(C53,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C53), "", RANK(C53,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>
@@ -6637,7 +6533,7 @@
         <v>13862.23</v>
       </c>
       <c r="D54" s="44">
-        <f>RANK(C54,$C$3:$C$54,0)</f>
+        <f>IF(ISBLANK(C54), "", RANK(C54,$C$3:$C$54,0))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(excel): resolve nulos count, sumproduct div/0, date formatting and max date evaluation
</commit_message>
<xml_diff>
--- a/docs/examples/excel/cheatsheet_excel.xlsx
+++ b/docs/examples/excel/cheatsheet_excel.xlsx
@@ -22,12 +22,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="DD/MM/YYYY HH:MM"/>
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="DD/MM/YYYY HH:MM"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -198,7 +199,7 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -209,7 +210,7 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -224,7 +225,7 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -244,10 +245,10 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -271,7 +272,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -735,10 +736,8 @@
       <c r="F3" s="5" t="n">
         <v>2955.07</v>
       </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>2021-01-31</t>
-        </is>
+      <c r="G3" s="6" t="n">
+        <v>44227</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
@@ -778,10 +777,8 @@
       <c r="F4" s="10" t="n">
         <v>4842.67</v>
       </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>2020-06-14</t>
-        </is>
+      <c r="G4" s="11" t="n">
+        <v>43996</v>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
@@ -825,10 +822,8 @@
       <c r="F5" s="5" t="n">
         <v>8303.389999999999</v>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>2018-01-27</t>
-        </is>
+      <c r="G5" s="6" t="n">
+        <v>43127</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -872,10 +867,8 @@
       <c r="F6" s="10" t="n">
         <v>4102.85</v>
       </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>2019-02-01</t>
-        </is>
+      <c r="G6" s="11" t="n">
+        <v>43497</v>
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
@@ -917,10 +910,8 @@
         </is>
       </c>
       <c r="F7" s="4" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>2025-01-18</t>
-        </is>
+      <c r="G7" s="6" t="n">
+        <v>45675</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -964,10 +955,8 @@
       <c r="F8" s="10" t="n">
         <v>9059.57</v>
       </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>2019-02-18</t>
-        </is>
+      <c r="G8" s="11" t="n">
+        <v>43514</v>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
@@ -1011,10 +1000,8 @@
       <c r="F9" s="5" t="n">
         <v>7459.35</v>
       </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>2019-12-02</t>
-        </is>
+      <c r="G9" s="6" t="n">
+        <v>43801</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -1027,7 +1014,7 @@
         </is>
       </c>
       <c r="K9" s="8">
-        <f>COUNTA(F3:F54)-COUNT(F3:F54)</f>
+        <f>COUNTBLANK(F3:F54)</f>
         <v/>
       </c>
     </row>
@@ -1056,10 +1043,8 @@
         </is>
       </c>
       <c r="F10" s="9" t="n"/>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>2018-08-18</t>
-        </is>
+      <c r="G10" s="11" t="n">
+        <v>43330</v>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
@@ -1094,10 +1079,8 @@
       <c r="F11" s="5" t="n">
         <v>4701.01</v>
       </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>2023-08-07</t>
-        </is>
+      <c r="G11" s="6" t="n">
+        <v>45145</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -1130,10 +1113,8 @@
         </is>
       </c>
       <c r="F12" s="9" t="n"/>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>2022-06-24</t>
-        </is>
+      <c r="G12" s="11" t="n">
+        <v>44736</v>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
@@ -1168,10 +1149,8 @@
       <c r="F13" s="5" t="n">
         <v>7710.89</v>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>2022-09-26</t>
-        </is>
+      <c r="G13" s="6" t="n">
+        <v>44830</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -1206,10 +1185,8 @@
       <c r="F14" s="10" t="n">
         <v>13862.23</v>
       </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>2024-01-09</t>
-        </is>
+      <c r="G14" s="11" t="n">
+        <v>45300</v>
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
@@ -1244,10 +1221,8 @@
       <c r="F15" s="5" t="n">
         <v>8825.709999999999</v>
       </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>2020-01-02</t>
-        </is>
+      <c r="G15" s="6" t="n">
+        <v>43832</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -1282,10 +1257,8 @@
       <c r="F16" s="10" t="n">
         <v>9862.6</v>
       </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>2024-01-19</t>
-        </is>
+      <c r="G16" s="11" t="n">
+        <v>45310</v>
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
@@ -1318,10 +1291,8 @@
         </is>
       </c>
       <c r="F17" s="4" t="n"/>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>2020-09-13</t>
-        </is>
+      <c r="G17" s="6" t="n">
+        <v>44087</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -1356,10 +1327,8 @@
       <c r="F18" s="10" t="n">
         <v>8937.76</v>
       </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>2024-03-01</t>
-        </is>
+      <c r="G18" s="11" t="n">
+        <v>45352</v>
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
@@ -1394,10 +1363,8 @@
       <c r="F19" s="5" t="n">
         <v>7220.28</v>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>2022-06-23</t>
-        </is>
+      <c r="G19" s="6" t="n">
+        <v>44735</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
@@ -1428,10 +1395,8 @@
       <c r="F20" s="10" t="n">
         <v>7324.01</v>
       </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>2020-07-31</t>
-        </is>
+      <c r="G20" s="11" t="n">
+        <v>44043</v>
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
@@ -1466,10 +1431,8 @@
       <c r="F21" s="5" t="n">
         <v>6842.01</v>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>2021-02-14</t>
-        </is>
+      <c r="G21" s="6" t="n">
+        <v>44241</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
@@ -1538,10 +1501,8 @@
       <c r="F23" s="5" t="n">
         <v>3175.8</v>
       </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>2021-10-21</t>
-        </is>
+      <c r="G23" s="6" t="n">
+        <v>44490</v>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
@@ -1608,10 +1569,8 @@
         </is>
       </c>
       <c r="F25" s="4" t="n"/>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>2023-06-13</t>
-        </is>
+      <c r="G25" s="6" t="n">
+        <v>45090</v>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
@@ -1646,10 +1605,8 @@
       <c r="F26" s="10" t="n">
         <v>9364.59</v>
       </c>
-      <c r="G26" s="11" t="inlineStr">
-        <is>
-          <t>2024-03-26</t>
-        </is>
+      <c r="G26" s="11" t="n">
+        <v>45377</v>
       </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
@@ -1684,10 +1641,8 @@
       <c r="F27" s="5" t="n">
         <v>8983.799999999999</v>
       </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>2018-08-23</t>
-        </is>
+      <c r="G27" s="6" t="n">
+        <v>43335</v>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
@@ -1722,10 +1677,8 @@
       <c r="F28" s="10" t="n">
         <v>5890.78</v>
       </c>
-      <c r="G28" s="11" t="inlineStr">
-        <is>
-          <t>2018-10-06</t>
-        </is>
+      <c r="G28" s="11" t="n">
+        <v>43379</v>
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
@@ -1760,10 +1713,8 @@
       <c r="F29" s="5" t="n">
         <v>10449.92</v>
       </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>2024-07-18</t>
-        </is>
+      <c r="G29" s="6" t="n">
+        <v>45491</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
@@ -1794,10 +1745,8 @@
       <c r="F30" s="10" t="n">
         <v>12224.44</v>
       </c>
-      <c r="G30" s="11" t="inlineStr">
-        <is>
-          <t>2021-05-13</t>
-        </is>
+      <c r="G30" s="11" t="n">
+        <v>44329</v>
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
@@ -1832,10 +1781,8 @@
       <c r="F31" s="5" t="n">
         <v>7047.08</v>
       </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>2019-06-27</t>
-        </is>
+      <c r="G31" s="6" t="n">
+        <v>43643</v>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
@@ -1870,10 +1817,8 @@
       <c r="F32" s="10" t="n">
         <v>6592.4</v>
       </c>
-      <c r="G32" s="11" t="inlineStr">
-        <is>
-          <t>2025-05-02</t>
-        </is>
+      <c r="G32" s="11" t="n">
+        <v>45779</v>
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
@@ -1908,10 +1853,8 @@
       <c r="F33" s="5" t="n">
         <v>14651.42</v>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>2019-09-29</t>
-        </is>
+      <c r="G33" s="6" t="n">
+        <v>43737</v>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
@@ -1942,10 +1885,8 @@
       <c r="F34" s="10" t="n">
         <v>5008.97</v>
       </c>
-      <c r="G34" s="11" t="inlineStr">
-        <is>
-          <t>2018-07-28</t>
-        </is>
+      <c r="G34" s="11" t="n">
+        <v>43309</v>
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
@@ -1972,10 +1913,8 @@
       <c r="F35" s="5" t="n">
         <v>8318</v>
       </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>2024-03-09</t>
-        </is>
+      <c r="G35" s="6" t="n">
+        <v>45360</v>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
@@ -2010,10 +1949,8 @@
       <c r="F36" s="10" t="n">
         <v>9676.76</v>
       </c>
-      <c r="G36" s="11" t="inlineStr">
-        <is>
-          <t>2024-07-13</t>
-        </is>
+      <c r="G36" s="11" t="n">
+        <v>45486</v>
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
@@ -2048,10 +1985,8 @@
       <c r="F37" s="5" t="n">
         <v>7730.99</v>
       </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>2020-10-19</t>
-        </is>
+      <c r="G37" s="6" t="n">
+        <v>44123</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
@@ -2086,10 +2021,8 @@
       <c r="F38" s="10" t="n">
         <v>10781.45</v>
       </c>
-      <c r="G38" s="11" t="inlineStr">
-        <is>
-          <t>2019-12-27</t>
-        </is>
+      <c r="G38" s="11" t="n">
+        <v>43826</v>
       </c>
       <c r="H38" s="9" t="inlineStr">
         <is>
@@ -2124,10 +2057,8 @@
       <c r="F39" s="5" t="n">
         <v>4454.2</v>
       </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>2019-03-19</t>
-        </is>
+      <c r="G39" s="6" t="n">
+        <v>43543</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
@@ -2158,10 +2089,8 @@
       <c r="F40" s="10" t="n">
         <v>4949</v>
       </c>
-      <c r="G40" s="11" t="inlineStr">
-        <is>
-          <t>2025-05-27</t>
-        </is>
+      <c r="G40" s="11" t="n">
+        <v>45804</v>
       </c>
       <c r="H40" s="9" t="inlineStr">
         <is>
@@ -2196,10 +2125,8 @@
       <c r="F41" s="5" t="n">
         <v>8436.139999999999</v>
       </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>2024-01-06</t>
-        </is>
+      <c r="G41" s="6" t="n">
+        <v>45297</v>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
@@ -2234,10 +2161,8 @@
       <c r="F42" s="10" t="n">
         <v>4204.62</v>
       </c>
-      <c r="G42" s="11" t="inlineStr">
-        <is>
-          <t>2022-11-15</t>
-        </is>
+      <c r="G42" s="11" t="n">
+        <v>44880</v>
       </c>
       <c r="H42" s="9" t="inlineStr">
         <is>
@@ -2272,10 +2197,8 @@
       <c r="F43" s="5" t="n">
         <v>3399.48</v>
       </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>2022-11-22</t>
-        </is>
+      <c r="G43" s="6" t="n">
+        <v>44887</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
@@ -2310,10 +2233,8 @@
       <c r="F44" s="10" t="n">
         <v>15412.06</v>
       </c>
-      <c r="G44" s="11" t="inlineStr">
-        <is>
-          <t>2021-09-14</t>
-        </is>
+      <c r="G44" s="11" t="n">
+        <v>44453</v>
       </c>
       <c r="H44" s="9" t="inlineStr">
         <is>
@@ -2348,10 +2269,8 @@
       <c r="F45" s="5" t="n">
         <v>10875.74</v>
       </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>2020-02-25</t>
-        </is>
+      <c r="G45" s="6" t="n">
+        <v>43886</v>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
@@ -2386,10 +2305,8 @@
       <c r="F46" s="10" t="n">
         <v>5431</v>
       </c>
-      <c r="G46" s="11" t="inlineStr">
-        <is>
-          <t>2020-05-10</t>
-        </is>
+      <c r="G46" s="11" t="n">
+        <v>43961</v>
       </c>
       <c r="H46" s="9" t="inlineStr">
         <is>
@@ -2424,10 +2341,8 @@
       <c r="F47" s="5" t="n">
         <v>9349.879999999999</v>
       </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>2019-11-27</t>
-        </is>
+      <c r="G47" s="6" t="n">
+        <v>43796</v>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
@@ -2496,10 +2411,8 @@
       <c r="F49" s="5" t="n">
         <v>12760.98</v>
       </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>2022-04-22</t>
-        </is>
+      <c r="G49" s="6" t="n">
+        <v>44673</v>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
@@ -2534,10 +2447,8 @@
       <c r="F50" s="10" t="n">
         <v>7844.93</v>
       </c>
-      <c r="G50" s="11" t="inlineStr">
-        <is>
-          <t>2023-10-23</t>
-        </is>
+      <c r="G50" s="11" t="n">
+        <v>45222</v>
       </c>
       <c r="H50" s="9" t="inlineStr">
         <is>
@@ -2572,10 +2483,8 @@
       <c r="F51" s="5" t="n">
         <v>8690.25</v>
       </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>2022-12-18</t>
-        </is>
+      <c r="G51" s="6" t="n">
+        <v>44913</v>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
@@ -2610,10 +2519,8 @@
       <c r="F52" s="10" t="n">
         <v>7480.7</v>
       </c>
-      <c r="G52" s="11" t="inlineStr">
-        <is>
-          <t>2020-10-09</t>
-        </is>
+      <c r="G52" s="11" t="n">
+        <v>44113</v>
       </c>
       <c r="H52" s="9" t="inlineStr">
         <is>
@@ -2646,10 +2553,8 @@
         </is>
       </c>
       <c r="F53" s="4" t="n"/>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>2025-01-18</t>
-        </is>
+      <c r="G53" s="6" t="n">
+        <v>45675</v>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
@@ -2684,10 +2589,8 @@
       <c r="F54" s="10" t="n">
         <v>13862.23</v>
       </c>
-      <c r="G54" s="11" t="inlineStr">
-        <is>
-          <t>2024-01-09</t>
-        </is>
+      <c r="G54" s="11" t="n">
+        <v>45300</v>
       </c>
       <c r="H54" s="9" t="inlineStr">
         <is>
@@ -2906,7 +2809,7 @@
         </is>
       </c>
       <c r="F10" s="18">
-        <f>SUMPRODUCT(1/COUNTIF(Dados!C3:C53,Dados!C3:C53))</f>
+        <f>SUMPRODUCT((Dados!C3:C54&lt;&gt;"")/COUNTIF(Dados!C3:C54,Dados!C3:C54&amp;""))</f>
         <v/>
       </c>
     </row>
@@ -3321,7 +3224,7 @@
           <t>Tempo de casa (dias)</t>
         </is>
       </c>
-      <c r="F3" s="32">
+      <c r="F3" s="17">
         <f>TODAY()-Dados!G3</f>
         <v/>
       </c>
@@ -3341,7 +3244,7 @@
           <t>Tempo de casa (anos)</t>
         </is>
       </c>
-      <c r="F4" s="33">
+      <c r="F4" s="32">
         <f>YEARFRAC(Dados!G3,TODAY())</f>
         <v/>
       </c>
@@ -3381,7 +3284,7 @@
           <t>Data + 30 dias</t>
         </is>
       </c>
-      <c r="F6" s="32">
+      <c r="F6" s="33">
         <f>Dados!G3+30</f>
         <v/>
       </c>
@@ -3401,7 +3304,7 @@
           <t>Primeiro dia do mes</t>
         </is>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="33">
         <f>DATE(YEAR(Dados!G3),MONTH(Dados!G3),1)</f>
         <v/>
       </c>
@@ -3421,7 +3324,7 @@
           <t>Ultimo dia do mes</t>
         </is>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="33">
         <f>EOMONTH(Dados!G3,0)</f>
         <v/>
       </c>
@@ -3441,7 +3344,7 @@
           <t>Dias entre duas datas</t>
         </is>
       </c>
-      <c r="F9" s="32">
+      <c r="F9" s="17">
         <f>_xlfn.DAYS(TODAY(),Dados!G3)</f>
         <v/>
       </c>
@@ -3461,7 +3364,7 @@
           <t>Dias uteis entre datas</t>
         </is>
       </c>
-      <c r="F10" s="32">
+      <c r="F10" s="17">
         <f>WORKDAY(Dados!G3,30)</f>
         <v/>
       </c>
@@ -3501,7 +3404,7 @@
           <t>Mais recente admissao</t>
         </is>
       </c>
-      <c r="F12" s="32">
+      <c r="F12" s="33">
         <f>MAX(Dados!G3:G54)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
fix(excel): generate final version of excel with workday formatting and description
</commit_message>
<xml_diff>
--- a/docs/examples/excel/cheatsheet_excel.xlsx
+++ b/docs/examples/excel/cheatsheet_excel.xlsx
@@ -3361,10 +3361,10 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>Dias uteis entre datas</t>
-        </is>
-      </c>
-      <c r="F10" s="17">
+          <t>Data + 30 dias uteis</t>
+        </is>
+      </c>
+      <c r="F10" s="33">
         <f>WORKDAY(Dados!G3,30)</f>
         <v/>
       </c>

</xml_diff>